<commit_message>
Ensure that KIA unit is buttoned up during a collateral attack. Fix type in Rules.xlsx. Change EventViewer.Show_CollateralDamageResults()  to check for collateral damage if number greater than one. Remove checking for CollateralDamage in ShowFriendlyActionResults()
</commit_message>
<xml_diff>
--- a/DesignDocs/Rules.xlsx
+++ b/DesignDocs/Rules.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cstewa01\source\repos\happysulla\PattonsBest\DesignDocs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cstew\source\repos\PattonsBest\DesignDocs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{1DC05E58-1CE6-43E0-9007-864EE9C449DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{7DEED4FA-5C24-4414-B243-AD5EB6D5155E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{89590866-6083-4176-8CBF-8C95C9BA24C2}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{89590866-6083-4176-8CBF-8C95C9BA24C2}"/>
   </bookViews>
   <sheets>
     <sheet name="Rules" sheetId="1" r:id="rId1"/>
@@ -3075,25 +3075,6 @@
 &lt;InlineUIContainer&gt;&lt;Button Content='r20.4' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; Counterattack Scenario&lt;LineBreak/&gt;</t>
   </si>
   <si>
-    <t>&lt;Bold&gt;r20.43 CounterAttack - Battle&lt;/Bold&gt;
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-When performing the Battle portion of a Counterattack sceanrio, delete steps &lt;InlineUIContainer&gt;&lt;Button Content='r4.61' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; and 
-&lt;InlineUIContainer&gt;&lt;Button Content='r4.64' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;. 
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;When rolling for Ambush per 
-&lt;InlineUIContainer&gt;&lt;Button Content='r4.65' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;, 
-if no Ambush occurs, go to the Battle Round Sequence 
-&lt;InlineUIContainer&gt;&lt;Button Content='r4.7' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;. If an Ambush does occur, do not conduct Enemy Actions, but instead perform the following steps:
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-For your tank, perform Battle Sequence &lt;InlineUIContainer&gt;&lt;Button Content='r4.72' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; -&gt; 
-&lt;InlineUIContainer&gt;&lt;Button Content='r4.74' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;&lt;LineBreak/&gt;
-Perform step &lt;InlineUIContainer&gt;&lt;Button Content='r4.76' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;: Friendly Action Phase &lt;LineBreak/&gt;
-Perform step &lt;InlineUIContainer&gt;&lt;Button Content='r4.77' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;: Random Events Phase&lt;LineBreak/&gt;
-Go to Battle Round Sequence &lt;InlineUIContainer&gt;&lt;Button Content='r4.7' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-If you clear the Battle Board, go to &lt;InlineUIContainer&gt;&lt;Button Content='r20.44' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; &lt;LineBreak/&gt;
-If you retreat from the Battle Board, go to &lt;InlineUIContainer&gt;&lt;Button Content='r20.45' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;</t>
-  </si>
-  <si>
     <t>&lt;Bold&gt;r4.61  Placement of Advancing Fire&lt;/Bold&gt;
 &lt;LineBreak/&gt;&lt;LineBreak/&gt;
 Place Advancing Fire markers per 
@@ -4035,6 +4016,25 @@
 Place the Sherman tank counter for the tank model you are using in the center of the Battle Board. If you want the turret to face a different sector than the tank itself, place a Turret marker on the tank counter accordingly.
 &lt;LineBreak/&gt;&lt;LineBreak/&gt;
                                      &lt;InlineUIContainer&gt;&lt;Image Name='c16TurretSherman75'  Height='100' Width='100'&gt;&lt;/Image&gt;&lt;/InlineUIContainer&gt;</t>
+  </si>
+  <si>
+    <t>&lt;Bold&gt;r20.43 CounterAttack - Battle&lt;/Bold&gt;
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+When performing the Battle portion of a Counterattack scenario, delete steps &lt;InlineUIContainer&gt;&lt;Button Content='r4.61' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; and 
+&lt;InlineUIContainer&gt;&lt;Button Content='r4.64' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;. 
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;When rolling for Ambush per 
+&lt;InlineUIContainer&gt;&lt;Button Content='r4.65' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;, 
+if no Ambush occurs, go to the Battle Round Sequence 
+&lt;InlineUIContainer&gt;&lt;Button Content='r4.7' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;. If an Ambush does occur, do not conduct Enemy Actions, but instead perform the following steps:
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+For your tank, perform Battle Sequence &lt;InlineUIContainer&gt;&lt;Button Content='r4.72' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; -&gt; 
+&lt;InlineUIContainer&gt;&lt;Button Content='r4.74' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;&lt;LineBreak/&gt;
+Perform step &lt;InlineUIContainer&gt;&lt;Button Content='r4.76' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;: Friendly Action Phase &lt;LineBreak/&gt;
+Perform step &lt;InlineUIContainer&gt;&lt;Button Content='r4.77' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;: Random Events Phase&lt;LineBreak/&gt;
+Go to Battle Round Sequence &lt;InlineUIContainer&gt;&lt;Button Content='r4.7' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+If you clear the Battle Board, go to &lt;InlineUIContainer&gt;&lt;Button Content='r20.44' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; &lt;LineBreak/&gt;
+If you retreat from the Battle Board, go to &lt;InlineUIContainer&gt;&lt;Button Content='r20.45' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;</t>
   </si>
 </sst>
 </file>
@@ -4419,7 +4419,7 @@
         <v>46</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>571</v>
+        <v>570</v>
       </c>
     </row>
     <row r="2" spans="1:2" ht="91.7" customHeight="1" x14ac:dyDescent="0.25">
@@ -4451,7 +4451,7 @@
         <v>17</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>572</v>
+        <v>571</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="120" x14ac:dyDescent="0.25">
@@ -4459,7 +4459,7 @@
         <v>18</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>565</v>
+        <v>564</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="45" x14ac:dyDescent="0.25">
@@ -4563,7 +4563,7 @@
         <v>89</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>597</v>
+        <v>596</v>
       </c>
     </row>
     <row r="20" spans="1:2" ht="120" x14ac:dyDescent="0.25">
@@ -4595,7 +4595,7 @@
         <v>125</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>586</v>
+        <v>585</v>
       </c>
     </row>
     <row r="24" spans="1:2" ht="120" x14ac:dyDescent="0.25">
@@ -4675,7 +4675,7 @@
         <v>225</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>501</v>
+        <v>500</v>
       </c>
     </row>
     <row r="34" spans="1:2" ht="165" x14ac:dyDescent="0.25">
@@ -4707,7 +4707,7 @@
         <v>229</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
     </row>
     <row r="38" spans="1:2" ht="135" x14ac:dyDescent="0.25">
@@ -4747,39 +4747,39 @@
         <v>441</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
     </row>
     <row r="43" spans="1:2" ht="105" x14ac:dyDescent="0.25">
       <c r="A43" s="5" t="s">
-        <v>521</v>
+        <v>520</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
     </row>
     <row r="44" spans="1:2" ht="285" x14ac:dyDescent="0.25">
       <c r="A44" s="5" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
     </row>
     <row r="45" spans="1:2" ht="135" x14ac:dyDescent="0.25">
       <c r="A45" s="5" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>531</v>
+        <v>530</v>
       </c>
     </row>
     <row r="46" spans="1:2" ht="210" x14ac:dyDescent="0.25">
       <c r="A46" s="5" t="s">
-        <v>524</v>
+        <v>523</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>581</v>
+        <v>580</v>
       </c>
     </row>
     <row r="47" spans="1:2" ht="300" x14ac:dyDescent="0.25">
@@ -4787,7 +4787,7 @@
         <v>442</v>
       </c>
       <c r="B47" s="2" t="s">
-        <v>503</v>
+        <v>502</v>
       </c>
     </row>
     <row r="48" spans="1:2" ht="150" x14ac:dyDescent="0.25">
@@ -4795,7 +4795,7 @@
         <v>443</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>512</v>
+        <v>511</v>
       </c>
     </row>
     <row r="49" spans="1:2" ht="180" x14ac:dyDescent="0.25">
@@ -4803,7 +4803,7 @@
         <v>444</v>
       </c>
       <c r="B49" s="2" t="s">
-        <v>513</v>
+        <v>512</v>
       </c>
     </row>
     <row r="50" spans="1:2" ht="60" x14ac:dyDescent="0.25">
@@ -4811,31 +4811,31 @@
         <v>445</v>
       </c>
       <c r="B50" s="2" t="s">
-        <v>517</v>
+        <v>516</v>
       </c>
     </row>
     <row r="51" spans="1:2" ht="240" x14ac:dyDescent="0.25">
       <c r="A51" s="5" t="s">
-        <v>514</v>
+        <v>513</v>
       </c>
       <c r="B51" s="2" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
     </row>
     <row r="52" spans="1:2" ht="390" x14ac:dyDescent="0.25">
       <c r="A52" s="5" t="s">
-        <v>516</v>
+        <v>515</v>
       </c>
       <c r="B52" s="2" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
     </row>
     <row r="53" spans="1:2" ht="195" x14ac:dyDescent="0.25">
       <c r="A53" s="5" t="s">
-        <v>515</v>
+        <v>514</v>
       </c>
       <c r="B53" s="2" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
     </row>
     <row r="54" spans="1:2" ht="105" x14ac:dyDescent="0.25">
@@ -4955,7 +4955,7 @@
         <v>208</v>
       </c>
       <c r="B68" s="2" t="s">
-        <v>573</v>
+        <v>572</v>
       </c>
     </row>
     <row r="69" spans="1:2" ht="135" x14ac:dyDescent="0.25">
@@ -4963,7 +4963,7 @@
         <v>209</v>
       </c>
       <c r="B69" s="2" t="s">
-        <v>507</v>
+        <v>506</v>
       </c>
     </row>
     <row r="70" spans="1:2" ht="90" x14ac:dyDescent="0.25">
@@ -4987,7 +4987,7 @@
         <v>190</v>
       </c>
       <c r="B72" s="2" t="s">
-        <v>585</v>
+        <v>584</v>
       </c>
     </row>
     <row r="73" spans="1:2" ht="195" x14ac:dyDescent="0.25">
@@ -5043,7 +5043,7 @@
         <v>263</v>
       </c>
       <c r="B79" s="2" t="s">
-        <v>582</v>
+        <v>581</v>
       </c>
     </row>
     <row r="80" spans="1:2" ht="135" x14ac:dyDescent="0.25">
@@ -5051,7 +5051,7 @@
         <v>264</v>
       </c>
       <c r="B80" s="2" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
     </row>
     <row r="81" spans="1:2" ht="120" x14ac:dyDescent="0.25">
@@ -5067,7 +5067,7 @@
         <v>266</v>
       </c>
       <c r="B82" s="2" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
     </row>
     <row r="83" spans="1:2" ht="135" x14ac:dyDescent="0.25">
@@ -5123,7 +5123,7 @@
         <v>273</v>
       </c>
       <c r="B89" s="2" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
     </row>
     <row r="90" spans="1:2" ht="90" x14ac:dyDescent="0.25">
@@ -5379,7 +5379,7 @@
         <v>343</v>
       </c>
       <c r="B121" s="2" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
     </row>
     <row r="122" spans="1:2" ht="120" x14ac:dyDescent="0.25">
@@ -5387,7 +5387,7 @@
         <v>335</v>
       </c>
       <c r="B122" s="2" t="s">
-        <v>527</v>
+        <v>526</v>
       </c>
     </row>
     <row r="123" spans="1:2" ht="90" x14ac:dyDescent="0.25">
@@ -5475,7 +5475,7 @@
         <v>368</v>
       </c>
       <c r="B133" s="2" t="s">
-        <v>576</v>
+        <v>575</v>
       </c>
     </row>
     <row r="134" spans="1:2" ht="90" x14ac:dyDescent="0.25">
@@ -5539,7 +5539,7 @@
         <v>381</v>
       </c>
       <c r="B141" s="2" t="s">
-        <v>588</v>
+        <v>587</v>
       </c>
     </row>
     <row r="142" spans="1:2" ht="165" x14ac:dyDescent="0.25">
@@ -5611,7 +5611,7 @@
         <v>232</v>
       </c>
       <c r="B150" s="2" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
     </row>
     <row r="151" spans="1:2" ht="195" x14ac:dyDescent="0.25">
@@ -5619,7 +5619,7 @@
         <v>233</v>
       </c>
       <c r="B151" s="2" t="s">
-        <v>592</v>
+        <v>591</v>
       </c>
     </row>
     <row r="152" spans="1:2" ht="225" x14ac:dyDescent="0.25">
@@ -5635,7 +5635,7 @@
         <v>235</v>
       </c>
       <c r="B153" s="2" t="s">
-        <v>577</v>
+        <v>576</v>
       </c>
     </row>
     <row r="154" spans="1:2" ht="75" x14ac:dyDescent="0.25">
@@ -5731,7 +5731,7 @@
         <v>364</v>
       </c>
       <c r="B165" s="2" t="s">
-        <v>563</v>
+        <v>562</v>
       </c>
     </row>
     <row r="166" spans="1:2" ht="195" x14ac:dyDescent="0.25">
@@ -5739,7 +5739,7 @@
         <v>408</v>
       </c>
       <c r="B166" s="2" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
     </row>
     <row r="167" spans="1:2" ht="75" x14ac:dyDescent="0.25">
@@ -5867,7 +5867,7 @@
         <v>404</v>
       </c>
       <c r="B182" s="2" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
     </row>
     <row r="183" spans="1:2" ht="105" x14ac:dyDescent="0.25">
@@ -5939,7 +5939,7 @@
         <v>77</v>
       </c>
       <c r="B191" s="2" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
     </row>
     <row r="192" spans="1:2" ht="120" x14ac:dyDescent="0.25">
@@ -5955,15 +5955,15 @@
         <v>79</v>
       </c>
       <c r="B193" s="2" t="s">
-        <v>530</v>
+        <v>529</v>
       </c>
     </row>
     <row r="194" spans="1:2" ht="60" x14ac:dyDescent="0.25">
       <c r="A194" s="5" t="s">
+        <v>527</v>
+      </c>
+      <c r="B194" s="2" t="s">
         <v>528</v>
-      </c>
-      <c r="B194" s="2" t="s">
-        <v>529</v>
       </c>
     </row>
     <row r="195" spans="1:2" ht="240" x14ac:dyDescent="0.25">
@@ -6059,7 +6059,7 @@
         <v>106</v>
       </c>
       <c r="B206" s="2" t="s">
-        <v>589</v>
+        <v>588</v>
       </c>
     </row>
     <row r="207" spans="1:2" ht="45" x14ac:dyDescent="0.25">
@@ -6075,7 +6075,7 @@
         <v>115</v>
       </c>
       <c r="B208" s="2" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
     </row>
     <row r="209" spans="1:2" ht="150" x14ac:dyDescent="0.25">
@@ -6091,7 +6091,7 @@
         <v>117</v>
       </c>
       <c r="B210" s="2" t="s">
-        <v>509</v>
+        <v>508</v>
       </c>
     </row>
     <row r="211" spans="1:2" ht="150" x14ac:dyDescent="0.25">
@@ -6099,7 +6099,7 @@
         <v>118</v>
       </c>
       <c r="B211" s="2" t="s">
-        <v>508</v>
+        <v>507</v>
       </c>
     </row>
     <row r="212" spans="1:2" ht="285" x14ac:dyDescent="0.25">
@@ -6171,7 +6171,7 @@
         <v>462</v>
       </c>
       <c r="B220" s="2" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
     </row>
     <row r="221" spans="1:2" ht="165" x14ac:dyDescent="0.25">
@@ -6179,7 +6179,7 @@
         <v>463</v>
       </c>
       <c r="B221" s="2" t="s">
-        <v>505</v>
+        <v>504</v>
       </c>
     </row>
     <row r="222" spans="1:2" ht="180" x14ac:dyDescent="0.25">
@@ -6187,7 +6187,7 @@
         <v>464</v>
       </c>
       <c r="B222" s="2" t="s">
-        <v>504</v>
+        <v>503</v>
       </c>
     </row>
     <row r="223" spans="1:2" ht="45" x14ac:dyDescent="0.25">
@@ -6395,7 +6395,7 @@
         <v>5</v>
       </c>
       <c r="B248" s="2" t="s">
-        <v>567</v>
+        <v>566</v>
       </c>
     </row>
     <row r="249" spans="1:2" ht="150" x14ac:dyDescent="0.25">
@@ -6403,7 +6403,7 @@
         <v>6</v>
       </c>
       <c r="B249" s="2" t="s">
-        <v>569</v>
+        <v>568</v>
       </c>
     </row>
     <row r="250" spans="1:2" ht="255" x14ac:dyDescent="0.25">
@@ -6411,7 +6411,7 @@
         <v>7</v>
       </c>
       <c r="B250" s="2" t="s">
-        <v>500</v>
+        <v>597</v>
       </c>
     </row>
     <row r="251" spans="1:2" ht="78.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -6419,7 +6419,7 @@
         <v>8</v>
       </c>
       <c r="B251" s="2" t="s">
-        <v>568</v>
+        <v>567</v>
       </c>
     </row>
     <row r="252" spans="1:2" ht="104.65" customHeight="1" x14ac:dyDescent="0.25">
@@ -6523,7 +6523,7 @@
         <v>156</v>
       </c>
       <c r="B264" s="3" t="s">
-        <v>511</v>
+        <v>510</v>
       </c>
     </row>
     <row r="265" spans="1:2" ht="165" x14ac:dyDescent="0.25">
@@ -6531,7 +6531,7 @@
         <v>159</v>
       </c>
       <c r="B265" s="3" t="s">
-        <v>510</v>
+        <v>509</v>
       </c>
     </row>
     <row r="266" spans="1:2" ht="165" x14ac:dyDescent="0.25">
@@ -6555,7 +6555,7 @@
         <v>488</v>
       </c>
       <c r="B268" s="3" t="s">
-        <v>596</v>
+        <v>595</v>
       </c>
     </row>
     <row r="269" spans="1:2" ht="150" x14ac:dyDescent="0.25">
@@ -6627,7 +6627,7 @@
         <v>481</v>
       </c>
       <c r="B277" s="3" t="s">
-        <v>593</v>
+        <v>592</v>
       </c>
     </row>
     <row r="278" spans="1:2" ht="105" x14ac:dyDescent="0.25">
@@ -6643,7 +6643,7 @@
         <v>483</v>
       </c>
       <c r="B279" s="3" t="s">
-        <v>595</v>
+        <v>594</v>
       </c>
     </row>
     <row r="280" spans="1:2" ht="120" x14ac:dyDescent="0.25">
@@ -6651,7 +6651,7 @@
         <v>485</v>
       </c>
       <c r="B280" s="3" t="s">
-        <v>566</v>
+        <v>565</v>
       </c>
     </row>
     <row r="281" spans="1:2" ht="105" x14ac:dyDescent="0.25">
@@ -6659,87 +6659,87 @@
         <v>486</v>
       </c>
       <c r="B281" s="3" t="s">
-        <v>594</v>
+        <v>593</v>
       </c>
     </row>
     <row r="282" spans="1:2" ht="270" x14ac:dyDescent="0.25">
       <c r="A282" s="1" t="s">
-        <v>542</v>
+        <v>541</v>
       </c>
       <c r="B282" s="3" t="s">
-        <v>557</v>
+        <v>556</v>
       </c>
     </row>
     <row r="283" spans="1:2" ht="150" x14ac:dyDescent="0.25">
       <c r="A283" s="1" t="s">
-        <v>543</v>
+        <v>542</v>
       </c>
       <c r="B283" s="3" t="s">
-        <v>552</v>
+        <v>551</v>
       </c>
     </row>
     <row r="284" spans="1:2" ht="60" x14ac:dyDescent="0.25">
       <c r="A284" s="1" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
       <c r="B284" s="3" t="s">
-        <v>558</v>
+        <v>557</v>
       </c>
     </row>
     <row r="285" spans="1:2" ht="60" x14ac:dyDescent="0.25">
       <c r="A285" s="1" t="s">
-        <v>545</v>
+        <v>544</v>
       </c>
       <c r="B285" s="3" t="s">
-        <v>553</v>
+        <v>552</v>
       </c>
     </row>
     <row r="286" spans="1:2" ht="60" x14ac:dyDescent="0.25">
       <c r="A286" s="1" t="s">
-        <v>546</v>
+        <v>545</v>
       </c>
       <c r="B286" s="3" t="s">
-        <v>555</v>
+        <v>554</v>
       </c>
     </row>
     <row r="287" spans="1:2" ht="60" x14ac:dyDescent="0.25">
       <c r="A287" s="1" t="s">
-        <v>547</v>
+        <v>546</v>
       </c>
       <c r="B287" s="3" t="s">
-        <v>554</v>
+        <v>553</v>
       </c>
     </row>
     <row r="288" spans="1:2" ht="60" x14ac:dyDescent="0.25">
       <c r="A288" s="1" t="s">
-        <v>548</v>
+        <v>547</v>
       </c>
       <c r="B288" s="3" t="s">
-        <v>556</v>
+        <v>555</v>
       </c>
     </row>
     <row r="289" spans="1:2" ht="60" x14ac:dyDescent="0.25">
       <c r="A289" s="1" t="s">
-        <v>549</v>
+        <v>548</v>
       </c>
       <c r="B289" s="3" t="s">
-        <v>559</v>
+        <v>558</v>
       </c>
     </row>
     <row r="290" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A290" s="1" t="s">
-        <v>550</v>
+        <v>549</v>
       </c>
       <c r="B290" s="3" t="s">
-        <v>560</v>
+        <v>559</v>
       </c>
     </row>
     <row r="291" spans="1:2" ht="195" x14ac:dyDescent="0.25">
       <c r="A291" s="1" t="s">
-        <v>551</v>
+        <v>550</v>
       </c>
       <c r="B291" s="3" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
     </row>
     <row r="292" spans="1:2" ht="180" x14ac:dyDescent="0.25">
@@ -6747,7 +6747,7 @@
         <v>493</v>
       </c>
       <c r="B292" s="3" t="s">
-        <v>587</v>
+        <v>586</v>
       </c>
     </row>
     <row r="293" spans="1:2" ht="120" x14ac:dyDescent="0.25">
@@ -6755,7 +6755,7 @@
         <v>494</v>
       </c>
       <c r="B293" s="3" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
     </row>
     <row r="294" spans="1:2" ht="135" x14ac:dyDescent="0.25">
@@ -6763,47 +6763,47 @@
         <v>495</v>
       </c>
       <c r="B294" s="3" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
     </row>
     <row r="295" spans="1:2" ht="210" x14ac:dyDescent="0.25">
       <c r="A295" s="1" t="s">
+        <v>532</v>
+      </c>
+      <c r="B295" s="3" t="s">
         <v>533</v>
-      </c>
-      <c r="B295" s="3" t="s">
-        <v>534</v>
       </c>
     </row>
     <row r="296" spans="1:2" ht="45" x14ac:dyDescent="0.25">
       <c r="A296" s="1" t="s">
-        <v>535</v>
+        <v>534</v>
       </c>
       <c r="B296" s="3" t="s">
-        <v>539</v>
+        <v>538</v>
       </c>
     </row>
     <row r="297" spans="1:2" ht="45" x14ac:dyDescent="0.25">
       <c r="A297" s="1" t="s">
-        <v>536</v>
+        <v>535</v>
       </c>
       <c r="B297" s="3" t="s">
-        <v>540</v>
+        <v>539</v>
       </c>
     </row>
     <row r="298" spans="1:2" ht="135" x14ac:dyDescent="0.25">
       <c r="A298" s="1" t="s">
-        <v>537</v>
+        <v>536</v>
       </c>
       <c r="B298" s="3" t="s">
-        <v>541</v>
+        <v>540</v>
       </c>
     </row>
     <row r="299" spans="1:2" ht="75" x14ac:dyDescent="0.25">
       <c r="A299" s="1" t="s">
-        <v>538</v>
+        <v>537</v>
       </c>
       <c r="B299" s="3" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="303" spans="1:2" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Make it clear in Rules.txt that MG use is only optional for non-digital games
</commit_message>
<xml_diff>
--- a/DesignDocs/Rules.xlsx
+++ b/DesignDocs/Rules.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cstew\source\repos\PattonsBest\DesignDocs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{7DEED4FA-5C24-4414-B243-AD5EB6D5155E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{9D6326A0-45E5-4D8B-B14D-B0125C409968}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{89590866-6083-4176-8CBF-8C95C9BA24C2}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{89590866-6083-4176-8CBF-8C95C9BA24C2}"/>
   </bookViews>
   <sheets>
     <sheet name="Rules" sheetId="1" r:id="rId1"/>
@@ -3377,11 +3377,6 @@
     <t>r16.3</t>
   </si>
   <si>
-    <t>&lt;Bold&gt;r16.3 Machine Gun (MG) Ammo (OPTIONAL)&lt;/Bold&gt; 
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-All rules dealing with MG ammunition should be considered optional and be followed only by choice. For most players, the additional problems posed by the consideration of MG ammo are not worth the record keeping involved. Continue to check for MG malfunctions, but otherwise assume there is sufficient MG ammo on hand for all firing.</t>
-  </si>
-  <si>
     <t>&lt;Bold&gt;r16.23 Ammo Ready Rack&lt;/Bold&gt; B5
 &lt;LineBreak/&gt;&lt;LineBreak/&gt;
 On the Tank Card, mark the number and types of rounds loaded into your ready rack with the Rounds Left markers. Reloading from the ready rack during battle increases the chance of achieving 
@@ -3894,20 +3889,6 @@
       &lt;InlineUIContainer&gt;&lt;Image Name='c35TaskForce'  Height='100' Width='100'&gt;&lt;/Image&gt;&lt;/InlineUIContainer&gt;</t>
   </si>
   <si>
-    <t>&lt;Bold&gt;r29.0 Fuel&lt;/Bold&gt;
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-All Sherman tank models carry a maxium of 35 units of fuel, where each unit equals 5 gallons (175 gallons total). During the Time Check step 
-&lt;InlineUIContainer&gt;&lt;Button Content='r4.3' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; of the sequence of play, when you determine the amount of time and ammo already expended for the day, 
-the number rolled also deteremines the number of fuel units already used.
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-Subtract the number rolled from 35 to determine the number of fuel units remaining. 
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-Thereafter, fuel is consumed for action on both the Movement and Battle Boards, and is subtracted from the remaining total with each use. 
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-&lt;InlineUIContainer&gt;&lt;Button Content='r29.1' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; Movement Board Fuel Use&lt;LineBreak/&gt;
-&lt;InlineUIContainer&gt;&lt;Button Content='r29.2' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; Battle Board Fuel Use</t>
-  </si>
-  <si>
     <t>&lt;Bold&gt;r11.11 Throwing a Track&lt;/Bold&gt; 
 &lt;LineBreak/&gt;&lt;LineBreak/&gt;
 A tank with a thrown track may not move or pivot for the remainder of the battle. Your tank sits where it is until it is knocked out or until all enemy units withdraw or are eliminated. Enemy units that are supposed to move are indicated with 'Do Nothing (TT)'.
@@ -4035,6 +4016,25 @@
 &lt;LineBreak/&gt;&lt;LineBreak/&gt;
 If you clear the Battle Board, go to &lt;InlineUIContainer&gt;&lt;Button Content='r20.44' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; &lt;LineBreak/&gt;
 If you retreat from the Battle Board, go to &lt;InlineUIContainer&gt;&lt;Button Content='r20.45' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;</t>
+  </si>
+  <si>
+    <t>&lt;Bold&gt;r16.3 Machine Gun (MG) Ammo (Only Optional if not using digital game)&lt;/Bold&gt; 
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+All rules dealing with MG ammunition should be considered optional and be followed only by choice. For most players, the additional problems posed by the consideration of MG ammo are not worth the record keeping involved. Continue to check for MG malfunctions, but otherwise assume there is sufficient MG ammo on hand for all firing.</t>
+  </si>
+  <si>
+    <t>&lt;Bold&gt;r29.0 Fuel (Only Optional if not using digital game)&lt;/Bold&gt;
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+All Sherman tank models carry a maxium of 35 units of fuel, where each unit equals 5 gallons (175 gallons total). During the Time Check step 
+&lt;InlineUIContainer&gt;&lt;Button Content='r4.3' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; of the sequence of play, when you determine the amount of time and ammo already expended for the day, 
+the number rolled also deteremines the number of fuel units already used.
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+Subtract the number rolled from 35 to determine the number of fuel units remaining. 
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+Thereafter, fuel is consumed for action on both the Movement and Battle Boards, and is subtracted from the remaining total with each use. 
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+&lt;InlineUIContainer&gt;&lt;Button Content='r29.1' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; Movement Board Fuel Use&lt;LineBreak/&gt;
+&lt;InlineUIContainer&gt;&lt;Button Content='r29.2' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; Battle Board Fuel Use</t>
   </si>
 </sst>
 </file>
@@ -4419,7 +4419,7 @@
         <v>46</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
     </row>
     <row r="2" spans="1:2" ht="91.7" customHeight="1" x14ac:dyDescent="0.25">
@@ -4451,7 +4451,7 @@
         <v>17</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>571</v>
+        <v>570</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="120" x14ac:dyDescent="0.25">
@@ -4459,7 +4459,7 @@
         <v>18</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="45" x14ac:dyDescent="0.25">
@@ -4563,7 +4563,7 @@
         <v>89</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>596</v>
+        <v>594</v>
       </c>
     </row>
     <row r="20" spans="1:2" ht="120" x14ac:dyDescent="0.25">
@@ -4595,7 +4595,7 @@
         <v>125</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>585</v>
+        <v>584</v>
       </c>
     </row>
     <row r="24" spans="1:2" ht="120" x14ac:dyDescent="0.25">
@@ -4763,7 +4763,7 @@
         <v>521</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>531</v>
+        <v>530</v>
       </c>
     </row>
     <row r="45" spans="1:2" ht="135" x14ac:dyDescent="0.25">
@@ -4771,7 +4771,7 @@
         <v>522</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>530</v>
+        <v>529</v>
       </c>
     </row>
     <row r="46" spans="1:2" ht="210" x14ac:dyDescent="0.25">
@@ -4779,7 +4779,7 @@
         <v>523</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
     </row>
     <row r="47" spans="1:2" ht="300" x14ac:dyDescent="0.25">
@@ -4955,7 +4955,7 @@
         <v>208</v>
       </c>
       <c r="B68" s="2" t="s">
-        <v>572</v>
+        <v>571</v>
       </c>
     </row>
     <row r="69" spans="1:2" ht="135" x14ac:dyDescent="0.25">
@@ -4987,7 +4987,7 @@
         <v>190</v>
       </c>
       <c r="B72" s="2" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
     </row>
     <row r="73" spans="1:2" ht="195" x14ac:dyDescent="0.25">
@@ -5043,7 +5043,7 @@
         <v>263</v>
       </c>
       <c r="B79" s="2" t="s">
-        <v>581</v>
+        <v>580</v>
       </c>
     </row>
     <row r="80" spans="1:2" ht="135" x14ac:dyDescent="0.25">
@@ -5051,7 +5051,7 @@
         <v>264</v>
       </c>
       <c r="B80" s="2" t="s">
-        <v>582</v>
+        <v>581</v>
       </c>
     </row>
     <row r="81" spans="1:2" ht="120" x14ac:dyDescent="0.25">
@@ -5067,7 +5067,7 @@
         <v>266</v>
       </c>
       <c r="B82" s="2" t="s">
-        <v>569</v>
+        <v>568</v>
       </c>
     </row>
     <row r="83" spans="1:2" ht="135" x14ac:dyDescent="0.25">
@@ -5123,7 +5123,7 @@
         <v>273</v>
       </c>
       <c r="B89" s="2" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
     </row>
     <row r="90" spans="1:2" ht="90" x14ac:dyDescent="0.25">
@@ -5379,7 +5379,7 @@
         <v>343</v>
       </c>
       <c r="B121" s="2" t="s">
-        <v>577</v>
+        <v>576</v>
       </c>
     </row>
     <row r="122" spans="1:2" ht="120" x14ac:dyDescent="0.25">
@@ -5475,7 +5475,7 @@
         <v>368</v>
       </c>
       <c r="B133" s="2" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
     </row>
     <row r="134" spans="1:2" ht="90" x14ac:dyDescent="0.25">
@@ -5539,7 +5539,7 @@
         <v>381</v>
       </c>
       <c r="B141" s="2" t="s">
-        <v>587</v>
+        <v>585</v>
       </c>
     </row>
     <row r="142" spans="1:2" ht="165" x14ac:dyDescent="0.25">
@@ -5611,7 +5611,7 @@
         <v>232</v>
       </c>
       <c r="B150" s="2" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
     </row>
     <row r="151" spans="1:2" ht="195" x14ac:dyDescent="0.25">
@@ -5619,7 +5619,7 @@
         <v>233</v>
       </c>
       <c r="B151" s="2" t="s">
-        <v>591</v>
+        <v>589</v>
       </c>
     </row>
     <row r="152" spans="1:2" ht="225" x14ac:dyDescent="0.25">
@@ -5635,7 +5635,7 @@
         <v>235</v>
       </c>
       <c r="B153" s="2" t="s">
-        <v>576</v>
+        <v>575</v>
       </c>
     </row>
     <row r="154" spans="1:2" ht="75" x14ac:dyDescent="0.25">
@@ -5731,7 +5731,7 @@
         <v>364</v>
       </c>
       <c r="B165" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="166" spans="1:2" ht="195" x14ac:dyDescent="0.25">
@@ -5739,7 +5739,7 @@
         <v>408</v>
       </c>
       <c r="B166" s="2" t="s">
-        <v>563</v>
+        <v>562</v>
       </c>
     </row>
     <row r="167" spans="1:2" ht="75" x14ac:dyDescent="0.25">
@@ -5867,7 +5867,7 @@
         <v>404</v>
       </c>
       <c r="B182" s="2" t="s">
-        <v>590</v>
+        <v>588</v>
       </c>
     </row>
     <row r="183" spans="1:2" ht="105" x14ac:dyDescent="0.25">
@@ -5939,7 +5939,7 @@
         <v>77</v>
       </c>
       <c r="B191" s="2" t="s">
-        <v>573</v>
+        <v>572</v>
       </c>
     </row>
     <row r="192" spans="1:2" ht="120" x14ac:dyDescent="0.25">
@@ -5955,7 +5955,7 @@
         <v>79</v>
       </c>
       <c r="B193" s="2" t="s">
-        <v>529</v>
+        <v>528</v>
       </c>
     </row>
     <row r="194" spans="1:2" ht="60" x14ac:dyDescent="0.25">
@@ -5963,7 +5963,7 @@
         <v>527</v>
       </c>
       <c r="B194" s="2" t="s">
-        <v>528</v>
+        <v>596</v>
       </c>
     </row>
     <row r="195" spans="1:2" ht="240" x14ac:dyDescent="0.25">
@@ -6059,7 +6059,7 @@
         <v>106</v>
       </c>
       <c r="B206" s="2" t="s">
-        <v>588</v>
+        <v>586</v>
       </c>
     </row>
     <row r="207" spans="1:2" ht="45" x14ac:dyDescent="0.25">
@@ -6075,7 +6075,7 @@
         <v>115</v>
       </c>
       <c r="B208" s="2" t="s">
-        <v>589</v>
+        <v>587</v>
       </c>
     </row>
     <row r="209" spans="1:2" ht="150" x14ac:dyDescent="0.25">
@@ -6395,7 +6395,7 @@
         <v>5</v>
       </c>
       <c r="B248" s="2" t="s">
-        <v>566</v>
+        <v>565</v>
       </c>
     </row>
     <row r="249" spans="1:2" ht="150" x14ac:dyDescent="0.25">
@@ -6403,7 +6403,7 @@
         <v>6</v>
       </c>
       <c r="B249" s="2" t="s">
-        <v>568</v>
+        <v>567</v>
       </c>
     </row>
     <row r="250" spans="1:2" ht="255" x14ac:dyDescent="0.25">
@@ -6411,7 +6411,7 @@
         <v>7</v>
       </c>
       <c r="B250" s="2" t="s">
-        <v>597</v>
+        <v>595</v>
       </c>
     </row>
     <row r="251" spans="1:2" ht="78.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -6419,7 +6419,7 @@
         <v>8</v>
       </c>
       <c r="B251" s="2" t="s">
-        <v>567</v>
+        <v>566</v>
       </c>
     </row>
     <row r="252" spans="1:2" ht="104.65" customHeight="1" x14ac:dyDescent="0.25">
@@ -6555,7 +6555,7 @@
         <v>488</v>
       </c>
       <c r="B268" s="3" t="s">
-        <v>595</v>
+        <v>593</v>
       </c>
     </row>
     <row r="269" spans="1:2" ht="150" x14ac:dyDescent="0.25">
@@ -6627,7 +6627,7 @@
         <v>481</v>
       </c>
       <c r="B277" s="3" t="s">
-        <v>592</v>
+        <v>590</v>
       </c>
     </row>
     <row r="278" spans="1:2" ht="105" x14ac:dyDescent="0.25">
@@ -6643,7 +6643,7 @@
         <v>483</v>
       </c>
       <c r="B279" s="3" t="s">
-        <v>594</v>
+        <v>592</v>
       </c>
     </row>
     <row r="280" spans="1:2" ht="120" x14ac:dyDescent="0.25">
@@ -6651,7 +6651,7 @@
         <v>485</v>
       </c>
       <c r="B280" s="3" t="s">
-        <v>565</v>
+        <v>564</v>
       </c>
     </row>
     <row r="281" spans="1:2" ht="105" x14ac:dyDescent="0.25">
@@ -6659,87 +6659,87 @@
         <v>486</v>
       </c>
       <c r="B281" s="3" t="s">
-        <v>593</v>
+        <v>591</v>
       </c>
     </row>
     <row r="282" spans="1:2" ht="270" x14ac:dyDescent="0.25">
       <c r="A282" s="1" t="s">
-        <v>541</v>
+        <v>540</v>
       </c>
       <c r="B282" s="3" t="s">
-        <v>556</v>
+        <v>555</v>
       </c>
     </row>
     <row r="283" spans="1:2" ht="150" x14ac:dyDescent="0.25">
       <c r="A283" s="1" t="s">
-        <v>542</v>
+        <v>541</v>
       </c>
       <c r="B283" s="3" t="s">
-        <v>551</v>
+        <v>550</v>
       </c>
     </row>
     <row r="284" spans="1:2" ht="60" x14ac:dyDescent="0.25">
       <c r="A284" s="1" t="s">
-        <v>543</v>
+        <v>542</v>
       </c>
       <c r="B284" s="3" t="s">
-        <v>557</v>
+        <v>556</v>
       </c>
     </row>
     <row r="285" spans="1:2" ht="60" x14ac:dyDescent="0.25">
       <c r="A285" s="1" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
       <c r="B285" s="3" t="s">
-        <v>552</v>
+        <v>551</v>
       </c>
     </row>
     <row r="286" spans="1:2" ht="60" x14ac:dyDescent="0.25">
       <c r="A286" s="1" t="s">
-        <v>545</v>
+        <v>544</v>
       </c>
       <c r="B286" s="3" t="s">
-        <v>554</v>
+        <v>553</v>
       </c>
     </row>
     <row r="287" spans="1:2" ht="60" x14ac:dyDescent="0.25">
       <c r="A287" s="1" t="s">
-        <v>546</v>
+        <v>545</v>
       </c>
       <c r="B287" s="3" t="s">
-        <v>553</v>
+        <v>552</v>
       </c>
     </row>
     <row r="288" spans="1:2" ht="60" x14ac:dyDescent="0.25">
       <c r="A288" s="1" t="s">
-        <v>547</v>
+        <v>546</v>
       </c>
       <c r="B288" s="3" t="s">
-        <v>555</v>
+        <v>554</v>
       </c>
     </row>
     <row r="289" spans="1:2" ht="60" x14ac:dyDescent="0.25">
       <c r="A289" s="1" t="s">
-        <v>548</v>
+        <v>547</v>
       </c>
       <c r="B289" s="3" t="s">
-        <v>558</v>
+        <v>557</v>
       </c>
     </row>
     <row r="290" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A290" s="1" t="s">
-        <v>549</v>
+        <v>548</v>
       </c>
       <c r="B290" s="3" t="s">
-        <v>559</v>
+        <v>558</v>
       </c>
     </row>
     <row r="291" spans="1:2" ht="195" x14ac:dyDescent="0.25">
       <c r="A291" s="1" t="s">
-        <v>550</v>
+        <v>549</v>
       </c>
       <c r="B291" s="3" t="s">
-        <v>560</v>
+        <v>559</v>
       </c>
     </row>
     <row r="292" spans="1:2" ht="180" x14ac:dyDescent="0.25">
@@ -6747,7 +6747,7 @@
         <v>493</v>
       </c>
       <c r="B292" s="3" t="s">
-        <v>586</v>
+        <v>597</v>
       </c>
     </row>
     <row r="293" spans="1:2" ht="120" x14ac:dyDescent="0.25">
@@ -6755,7 +6755,7 @@
         <v>494</v>
       </c>
       <c r="B293" s="3" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
     </row>
     <row r="294" spans="1:2" ht="135" x14ac:dyDescent="0.25">
@@ -6763,47 +6763,47 @@
         <v>495</v>
       </c>
       <c r="B294" s="3" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
     </row>
     <row r="295" spans="1:2" ht="210" x14ac:dyDescent="0.25">
       <c r="A295" s="1" t="s">
+        <v>531</v>
+      </c>
+      <c r="B295" s="3" t="s">
         <v>532</v>
-      </c>
-      <c r="B295" s="3" t="s">
-        <v>533</v>
       </c>
     </row>
     <row r="296" spans="1:2" ht="45" x14ac:dyDescent="0.25">
       <c r="A296" s="1" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="B296" s="3" t="s">
-        <v>538</v>
+        <v>537</v>
       </c>
     </row>
     <row r="297" spans="1:2" ht="45" x14ac:dyDescent="0.25">
       <c r="A297" s="1" t="s">
-        <v>535</v>
+        <v>534</v>
       </c>
       <c r="B297" s="3" t="s">
-        <v>539</v>
+        <v>538</v>
       </c>
     </row>
     <row r="298" spans="1:2" ht="135" x14ac:dyDescent="0.25">
       <c r="A298" s="1" t="s">
-        <v>536</v>
+        <v>535</v>
       </c>
       <c r="B298" s="3" t="s">
-        <v>540</v>
+        <v>539</v>
       </c>
     </row>
     <row r="299" spans="1:2" ht="75" x14ac:dyDescent="0.25">
       <c r="A299" s="1" t="s">
-        <v>537</v>
+        <v>536</v>
       </c>
       <c r="B299" s="3" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
     </row>
     <row r="303" spans="1:2" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Show optional rule for MG fire
</commit_message>
<xml_diff>
--- a/DesignDocs/Rules.xlsx
+++ b/DesignDocs/Rules.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cstew\source\repos\PattonsBest\DesignDocs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{9D6326A0-45E5-4D8B-B14D-B0125C409968}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{9F78F578-95E3-4BE6-9A0E-7206975CEEF2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{89590866-6083-4176-8CBF-8C95C9BA24C2}"/>
   </bookViews>
@@ -1483,18 +1483,6 @@
 There is no limit on the number of enemy units that may be placed in the same sector, at the same range, and in the same terrain.</t>
   </si>
   <si>
-    <t>&lt;Bold&gt;r16.0 Ammunition (Ammo)&lt;/Bold&gt; 
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-Ammo is loaded into your tank at the beginning of each scenerio as part of morning briefing 
-&lt;InlineUIContainer&gt;&lt;Button Content='r4.2' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;. 
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-Each model and variant of the Sherman tank has a limit on its normal load and ammo, both for its man gun and MGs as shown on it Tank Card .  
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-&lt;InlineUIContainer&gt;&lt;Button Content='r16.0a' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; Details&lt;LineBreak/&gt;
-&lt;InlineUIContainer&gt;&lt;Button Content='r16.1' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;  Ammo Types&lt;LineBreak/&gt;
-&lt;InlineUIContainer&gt;&lt;Button Content='r16.2' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;  Loading Ammo</t>
-  </si>
-  <si>
     <t>&lt;Bold&gt;r12.14 Panzerspahwagen (PSW)&lt;/Bold&gt; 
 &lt;LineBreak/&gt;&lt;LineBreak/&gt;
 Armored scout car.
@@ -4018,12 +4006,25 @@
 If you retreat from the Battle Board, go to &lt;InlineUIContainer&gt;&lt;Button Content='r20.45' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;</t>
   </si>
   <si>
-    <t>&lt;Bold&gt;r16.3 Machine Gun (MG) Ammo (Only Optional if not using digital game)&lt;/Bold&gt; 
+    <t>&lt;Bold&gt;r16.0 Ammunition (Ammo)&lt;/Bold&gt; 
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+Ammo is loaded into your tank at the beginning of each scenerio as part of morning briefing 
+&lt;InlineUIContainer&gt;&lt;Button Content='r4.2' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;. 
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+Each model and variant of the Sherman tank has a limit on its normal load and ammo, both for its man gun and MGs as shown on it Tank Card .  
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+&lt;InlineUIContainer&gt;&lt;Button Content='r16.0a' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; Details&lt;LineBreak/&gt;
+&lt;InlineUIContainer&gt;&lt;Button Content='r16.1' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;  Ammo Types&lt;LineBreak/&gt;
+&lt;InlineUIContainer&gt;&lt;Button Content='r16.2' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;  Loading Ammo&lt;LineBreak/&gt;
+&lt;InlineUIContainer&gt;&lt;Button Content='r16.3' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; Machine Gun (MG) Ammo (Only Optional if not Using Digital Game)</t>
+  </si>
+  <si>
+    <t>&lt;Bold&gt;r16.3 Machine Gun (MG) Ammo (Only Optional if not Using Digital Game)&lt;/Bold&gt; 
 &lt;LineBreak/&gt;&lt;LineBreak/&gt;
 All rules dealing with MG ammunition should be considered optional and be followed only by choice. For most players, the additional problems posed by the consideration of MG ammo are not worth the record keeping involved. Continue to check for MG malfunctions, but otherwise assume there is sufficient MG ammo on hand for all firing.</t>
   </si>
   <si>
-    <t>&lt;Bold&gt;r29.0 Fuel (Only Optional if not using digital game)&lt;/Bold&gt;
+    <t>&lt;Bold&gt;r29.0 Fuel (Only Optional if not Using Digital Game)&lt;/Bold&gt;
 &lt;LineBreak/&gt;&lt;LineBreak/&gt;
 All Sherman tank models carry a maxium of 35 units of fuel, where each unit equals 5 gallons (175 gallons total). During the Time Check step 
 &lt;InlineUIContainer&gt;&lt;Button Content='r4.3' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; of the sequence of play, when you determine the amount of time and ammo already expended for the day, 
@@ -4419,7 +4420,7 @@
         <v>46</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>569</v>
+        <v>568</v>
       </c>
     </row>
     <row r="2" spans="1:2" ht="91.7" customHeight="1" x14ac:dyDescent="0.25">
@@ -4451,7 +4452,7 @@
         <v>17</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="120" x14ac:dyDescent="0.25">
@@ -4459,7 +4460,7 @@
         <v>18</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>563</v>
+        <v>562</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="45" x14ac:dyDescent="0.25">
@@ -4491,7 +4492,7 @@
         <v>49</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
     </row>
     <row r="11" spans="1:2" ht="165" x14ac:dyDescent="0.25">
@@ -4563,7 +4564,7 @@
         <v>89</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>594</v>
+        <v>593</v>
       </c>
     </row>
     <row r="20" spans="1:2" ht="120" x14ac:dyDescent="0.25">
@@ -4595,7 +4596,7 @@
         <v>125</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
     </row>
     <row r="24" spans="1:2" ht="120" x14ac:dyDescent="0.25">
@@ -4635,7 +4636,7 @@
         <v>130</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>497</v>
+        <v>496</v>
       </c>
     </row>
     <row r="29" spans="1:2" ht="150" x14ac:dyDescent="0.25">
@@ -4643,7 +4644,7 @@
         <v>131</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
     </row>
     <row r="30" spans="1:2" ht="120" x14ac:dyDescent="0.25">
@@ -4651,7 +4652,7 @@
         <v>132</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>498</v>
+        <v>497</v>
       </c>
     </row>
     <row r="31" spans="1:2" ht="360" x14ac:dyDescent="0.25">
@@ -4675,7 +4676,7 @@
         <v>225</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>500</v>
+        <v>499</v>
       </c>
     </row>
     <row r="34" spans="1:2" ht="165" x14ac:dyDescent="0.25">
@@ -4707,135 +4708,135 @@
         <v>229</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>501</v>
+        <v>500</v>
       </c>
     </row>
     <row r="38" spans="1:2" ht="135" x14ac:dyDescent="0.25">
       <c r="A38" s="5" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
     </row>
     <row r="39" spans="1:2" ht="75" x14ac:dyDescent="0.25">
       <c r="A39" s="5" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
     </row>
     <row r="40" spans="1:2" ht="150" x14ac:dyDescent="0.25">
       <c r="A40" s="5" t="s">
-        <v>439</v>
+        <v>438</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
     </row>
     <row r="41" spans="1:2" ht="150" x14ac:dyDescent="0.25">
       <c r="A41" s="5" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>480</v>
+        <v>479</v>
       </c>
     </row>
     <row r="42" spans="1:2" ht="135" x14ac:dyDescent="0.25">
       <c r="A42" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
     </row>
     <row r="43" spans="1:2" ht="105" x14ac:dyDescent="0.25">
       <c r="A43" s="5" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>524</v>
+        <v>523</v>
       </c>
     </row>
     <row r="44" spans="1:2" ht="285" x14ac:dyDescent="0.25">
       <c r="A44" s="5" t="s">
-        <v>521</v>
+        <v>520</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>530</v>
+        <v>529</v>
       </c>
     </row>
     <row r="45" spans="1:2" ht="135" x14ac:dyDescent="0.25">
       <c r="A45" s="5" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>529</v>
+        <v>528</v>
       </c>
     </row>
     <row r="46" spans="1:2" ht="210" x14ac:dyDescent="0.25">
       <c r="A46" s="5" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
     </row>
     <row r="47" spans="1:2" ht="300" x14ac:dyDescent="0.25">
       <c r="A47" s="5" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="B47" s="2" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
     </row>
     <row r="48" spans="1:2" ht="150" x14ac:dyDescent="0.25">
       <c r="A48" s="5" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>511</v>
+        <v>510</v>
       </c>
     </row>
     <row r="49" spans="1:2" ht="180" x14ac:dyDescent="0.25">
       <c r="A49" s="5" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
       <c r="B49" s="2" t="s">
-        <v>512</v>
+        <v>511</v>
       </c>
     </row>
     <row r="50" spans="1:2" ht="60" x14ac:dyDescent="0.25">
       <c r="A50" s="5" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="B50" s="2" t="s">
-        <v>516</v>
+        <v>515</v>
       </c>
     </row>
     <row r="51" spans="1:2" ht="240" x14ac:dyDescent="0.25">
       <c r="A51" s="5" t="s">
-        <v>513</v>
+        <v>512</v>
       </c>
       <c r="B51" s="2" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
     </row>
     <row r="52" spans="1:2" ht="390" x14ac:dyDescent="0.25">
       <c r="A52" s="5" t="s">
-        <v>515</v>
+        <v>514</v>
       </c>
       <c r="B52" s="2" t="s">
-        <v>517</v>
+        <v>516</v>
       </c>
     </row>
     <row r="53" spans="1:2" ht="195" x14ac:dyDescent="0.25">
       <c r="A53" s="5" t="s">
-        <v>514</v>
+        <v>513</v>
       </c>
       <c r="B53" s="2" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
     </row>
     <row r="54" spans="1:2" ht="105" x14ac:dyDescent="0.25">
@@ -4851,7 +4852,7 @@
         <v>166</v>
       </c>
       <c r="B55" s="2" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
     </row>
     <row r="56" spans="1:2" ht="135" x14ac:dyDescent="0.25">
@@ -4955,7 +4956,7 @@
         <v>208</v>
       </c>
       <c r="B68" s="2" t="s">
-        <v>571</v>
+        <v>570</v>
       </c>
     </row>
     <row r="69" spans="1:2" ht="135" x14ac:dyDescent="0.25">
@@ -4963,7 +4964,7 @@
         <v>209</v>
       </c>
       <c r="B69" s="2" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
     </row>
     <row r="70" spans="1:2" ht="90" x14ac:dyDescent="0.25">
@@ -4987,7 +4988,7 @@
         <v>190</v>
       </c>
       <c r="B72" s="2" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
     </row>
     <row r="73" spans="1:2" ht="195" x14ac:dyDescent="0.25">
@@ -5040,562 +5041,562 @@
     </row>
     <row r="79" spans="1:2" ht="165" x14ac:dyDescent="0.25">
       <c r="A79" s="5" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="B79" s="2" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
     </row>
     <row r="80" spans="1:2" ht="135" x14ac:dyDescent="0.25">
       <c r="A80" s="5" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="B80" s="2" t="s">
-        <v>581</v>
+        <v>580</v>
       </c>
     </row>
     <row r="81" spans="1:2" ht="120" x14ac:dyDescent="0.25">
       <c r="A81" s="5" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="B81" s="2" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
     </row>
     <row r="82" spans="1:2" ht="135" x14ac:dyDescent="0.25">
       <c r="A82" s="5" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="B82" s="2" t="s">
-        <v>568</v>
+        <v>567</v>
       </c>
     </row>
     <row r="83" spans="1:2" ht="135" x14ac:dyDescent="0.25">
       <c r="A83" s="5" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="B83" s="2" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
     </row>
     <row r="84" spans="1:2" ht="75" x14ac:dyDescent="0.25">
       <c r="A84" s="5" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="B84" s="2" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
     </row>
     <row r="85" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A85" s="5" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="B85" s="2" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
     </row>
     <row r="86" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A86" s="5" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="B86" s="2" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
     </row>
     <row r="87" spans="1:2" ht="105" x14ac:dyDescent="0.25">
       <c r="A87" s="5" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="B87" s="2" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
     </row>
     <row r="88" spans="1:2" ht="135" x14ac:dyDescent="0.25">
       <c r="A88" s="5" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="B88" s="2" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
     </row>
     <row r="89" spans="1:2" ht="195" x14ac:dyDescent="0.25">
       <c r="A89" s="5" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="B89" s="2" t="s">
-        <v>582</v>
+        <v>581</v>
       </c>
     </row>
     <row r="90" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A90" s="5" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="B90" s="2" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
     </row>
     <row r="91" spans="1:2" ht="105" x14ac:dyDescent="0.25">
       <c r="A91" s="5" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="B91" s="2" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
     </row>
     <row r="92" spans="1:2" ht="105" x14ac:dyDescent="0.25">
       <c r="A92" s="5" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="B92" s="2" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
     </row>
     <row r="93" spans="1:2" ht="75" x14ac:dyDescent="0.25">
       <c r="A93" s="5" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="B93" s="2" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
     </row>
     <row r="94" spans="1:2" ht="75" x14ac:dyDescent="0.25">
       <c r="A94" s="5" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="B94" s="2" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
     </row>
     <row r="95" spans="1:2" ht="75" x14ac:dyDescent="0.25">
       <c r="A95" s="5" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="B95" s="2" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
     </row>
     <row r="96" spans="1:2" ht="150" x14ac:dyDescent="0.25">
       <c r="A96" s="5" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="B96" s="2" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
     </row>
     <row r="97" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A97" s="5" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="B97" s="2" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
     </row>
     <row r="98" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A98" s="5" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="B98" s="2" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
     </row>
     <row r="99" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A99" s="5" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="B99" s="2" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="100" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A100" s="5" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="B100" s="2" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
     </row>
     <row r="101" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A101" s="5" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="B101" s="2" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
     </row>
     <row r="102" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A102" s="5" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="B102" s="2" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
     </row>
     <row r="103" spans="1:2" ht="105" x14ac:dyDescent="0.25">
       <c r="A103" s="5" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="B103" s="2" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
     </row>
     <row r="104" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A104" s="5" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="B104" s="2" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
     </row>
     <row r="105" spans="1:2" ht="105" x14ac:dyDescent="0.25">
       <c r="A105" s="5" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="B105" s="2" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
     </row>
     <row r="106" spans="1:2" ht="120" x14ac:dyDescent="0.25">
       <c r="A106" s="5" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="B106" s="2" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
     </row>
     <row r="107" spans="1:2" ht="105" x14ac:dyDescent="0.25">
       <c r="A107" s="5" t="s">
+        <v>290</v>
+      </c>
+      <c r="B107" s="2" t="s">
         <v>291</v>
-      </c>
-      <c r="B107" s="2" t="s">
-        <v>292</v>
       </c>
     </row>
     <row r="108" spans="1:2" ht="135" x14ac:dyDescent="0.25">
       <c r="A108" s="5" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="B108" s="2" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
     </row>
     <row r="109" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A109" s="5" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="B109" s="2" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
     </row>
     <row r="110" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A110" s="5" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="B110" s="2" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
     </row>
     <row r="111" spans="1:2" ht="75" x14ac:dyDescent="0.25">
       <c r="A111" s="5" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="B111" s="2" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
     </row>
     <row r="112" spans="1:2" ht="105" x14ac:dyDescent="0.25">
       <c r="A112" s="5" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="B112" s="2" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
     </row>
     <row r="113" spans="1:2" ht="255" x14ac:dyDescent="0.25">
       <c r="A113" s="5" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="B113" s="2" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
     </row>
     <row r="114" spans="1:2" ht="210" x14ac:dyDescent="0.25">
       <c r="A114" s="5" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="B114" s="2" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
     </row>
     <row r="115" spans="1:2" ht="135" x14ac:dyDescent="0.25">
       <c r="A115" s="5" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="B115" s="2" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
     </row>
     <row r="116" spans="1:2" ht="105" x14ac:dyDescent="0.25">
       <c r="A116" s="5" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="B116" s="2" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
     </row>
     <row r="117" spans="1:2" ht="120" x14ac:dyDescent="0.25">
       <c r="A117" s="5" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="B117" s="2" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
     </row>
     <row r="118" spans="1:2" ht="60" x14ac:dyDescent="0.25">
       <c r="A118" s="5" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="B118" s="2" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
     </row>
     <row r="119" spans="1:2" ht="135" x14ac:dyDescent="0.25">
       <c r="A119" s="5" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="B119" s="2" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
     </row>
     <row r="120" spans="1:2" ht="75" x14ac:dyDescent="0.25">
       <c r="A120" s="5" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="B120" s="2" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
     </row>
     <row r="121" spans="1:2" ht="195" x14ac:dyDescent="0.25">
       <c r="A121" s="5" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="B121" s="2" t="s">
-        <v>576</v>
+        <v>575</v>
       </c>
     </row>
     <row r="122" spans="1:2" ht="120" x14ac:dyDescent="0.25">
       <c r="A122" s="5" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="B122" s="2" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
     </row>
     <row r="123" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A123" s="5" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="B123" s="2" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
     </row>
     <row r="124" spans="1:2" ht="45" x14ac:dyDescent="0.25">
       <c r="A124" s="5" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="B124" s="2" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
     </row>
     <row r="125" spans="1:2" ht="105" x14ac:dyDescent="0.25">
       <c r="A125" s="5" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="B125" s="2" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
     </row>
     <row r="126" spans="1:2" ht="120" x14ac:dyDescent="0.25">
       <c r="A126" s="5" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="B126" s="2" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
     </row>
     <row r="127" spans="1:2" ht="180" x14ac:dyDescent="0.25">
       <c r="A127" s="5" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="B127" s="2" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
     </row>
     <row r="128" spans="1:2" ht="180" x14ac:dyDescent="0.25">
       <c r="A128" s="5" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="B128" s="2" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
     </row>
     <row r="129" spans="1:2" ht="60" x14ac:dyDescent="0.25">
       <c r="A129" s="5" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="B129" s="2" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
     </row>
     <row r="130" spans="1:2" ht="180" x14ac:dyDescent="0.25">
       <c r="A130" s="5" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="B130" s="2" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
     </row>
     <row r="131" spans="1:2" ht="285" x14ac:dyDescent="0.25">
       <c r="A131" s="5" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="B131" s="2" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
     </row>
     <row r="132" spans="1:2" ht="60" x14ac:dyDescent="0.25">
       <c r="A132" s="5" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="B132" s="2" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
     </row>
     <row r="133" spans="1:2" ht="195" x14ac:dyDescent="0.25">
       <c r="A133" s="5" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="B133" s="2" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
     </row>
     <row r="134" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A134" s="5" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="B134" s="2" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
     </row>
     <row r="135" spans="1:2" ht="75" x14ac:dyDescent="0.25">
       <c r="A135" s="5" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B135" s="2" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
     </row>
     <row r="136" spans="1:2" ht="135" x14ac:dyDescent="0.25">
       <c r="A136" s="5" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="B136" s="2" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
     </row>
     <row r="137" spans="1:2" ht="75" x14ac:dyDescent="0.25">
       <c r="A137" s="5" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="B137" s="2" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
     </row>
     <row r="138" spans="1:2" ht="180" x14ac:dyDescent="0.25">
       <c r="A138" s="5" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="B138" s="2" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
     </row>
     <row r="139" spans="1:2" ht="255" x14ac:dyDescent="0.25">
       <c r="A139" s="5" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="B139" s="2" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
     </row>
     <row r="140" spans="1:2" ht="210" x14ac:dyDescent="0.25">
       <c r="A140" s="5" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="B140" s="2" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
     </row>
     <row r="141" spans="1:2" ht="195" x14ac:dyDescent="0.25">
       <c r="A141" s="5" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="B141" s="2" t="s">
-        <v>585</v>
+        <v>584</v>
       </c>
     </row>
     <row r="142" spans="1:2" ht="165" x14ac:dyDescent="0.25">
       <c r="A142" s="5" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="B142" s="2" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
     </row>
     <row r="143" spans="1:2" ht="108.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A143" s="5" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="B143" s="2" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
     </row>
     <row r="144" spans="1:2" ht="210" x14ac:dyDescent="0.25">
       <c r="A144" s="5" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="B144" s="2" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
     </row>
     <row r="145" spans="1:2" ht="75" x14ac:dyDescent="0.25">
       <c r="A145" s="5" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="B145" s="2" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
     </row>
     <row r="146" spans="1:2" ht="75" x14ac:dyDescent="0.25">
       <c r="A146" s="5" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="B146" s="2" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
     </row>
     <row r="147" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A147" s="5" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="B147" s="2" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
     </row>
     <row r="148" spans="1:2" ht="105" x14ac:dyDescent="0.25">
       <c r="A148" s="5" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="B148" s="2" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
     </row>
     <row r="149" spans="1:2" ht="150" x14ac:dyDescent="0.25">
@@ -5611,7 +5612,7 @@
         <v>232</v>
       </c>
       <c r="B150" s="2" t="s">
-        <v>573</v>
+        <v>572</v>
       </c>
     </row>
     <row r="151" spans="1:2" ht="195" x14ac:dyDescent="0.25">
@@ -5619,7 +5620,7 @@
         <v>233</v>
       </c>
       <c r="B151" s="2" t="s">
-        <v>589</v>
+        <v>588</v>
       </c>
     </row>
     <row r="152" spans="1:2" ht="225" x14ac:dyDescent="0.25">
@@ -5627,7 +5628,7 @@
         <v>234</v>
       </c>
       <c r="B152" s="2" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
     </row>
     <row r="153" spans="1:2" ht="75" x14ac:dyDescent="0.25">
@@ -5635,7 +5636,7 @@
         <v>235</v>
       </c>
       <c r="B153" s="2" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
     </row>
     <row r="154" spans="1:2" ht="75" x14ac:dyDescent="0.25">
@@ -5643,7 +5644,7 @@
         <v>236</v>
       </c>
       <c r="B154" s="2" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
     </row>
     <row r="155" spans="1:2" ht="75" x14ac:dyDescent="0.25">
@@ -5651,7 +5652,7 @@
         <v>237</v>
       </c>
       <c r="B155" s="2" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
     </row>
     <row r="156" spans="1:2" ht="75" x14ac:dyDescent="0.25">
@@ -5659,7 +5660,7 @@
         <v>238</v>
       </c>
       <c r="B156" s="2" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
     </row>
     <row r="157" spans="1:2" ht="75" x14ac:dyDescent="0.25">
@@ -5667,7 +5668,7 @@
         <v>239</v>
       </c>
       <c r="B157" s="2" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
     </row>
     <row r="158" spans="1:2" ht="105" x14ac:dyDescent="0.25">
@@ -5675,7 +5676,7 @@
         <v>240</v>
       </c>
       <c r="B158" s="2" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
     </row>
     <row r="159" spans="1:2" ht="180" x14ac:dyDescent="0.25">
@@ -5707,7 +5708,7 @@
         <v>244</v>
       </c>
       <c r="B162" s="2" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
     </row>
     <row r="163" spans="1:2" ht="75" x14ac:dyDescent="0.25">
@@ -5715,7 +5716,7 @@
         <v>245</v>
       </c>
       <c r="B163" s="2" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="164" spans="1:2" ht="180" x14ac:dyDescent="0.25">
@@ -5723,191 +5724,191 @@
         <v>246</v>
       </c>
       <c r="B164" s="2" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
     </row>
     <row r="165" spans="1:2" ht="195" x14ac:dyDescent="0.25">
       <c r="A165" s="5" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="B165" s="2" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
     </row>
     <row r="166" spans="1:2" ht="195" x14ac:dyDescent="0.25">
       <c r="A166" s="5" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="B166" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="167" spans="1:2" ht="75" x14ac:dyDescent="0.25">
       <c r="A167" s="5" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="B167" s="2" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
     </row>
     <row r="168" spans="1:2" ht="75" x14ac:dyDescent="0.25">
       <c r="A168" s="5" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="B168" s="2" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
     </row>
     <row r="169" spans="1:2" ht="45" x14ac:dyDescent="0.25">
       <c r="A169" s="5" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="B169" s="2" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
     </row>
     <row r="170" spans="1:2" ht="45" x14ac:dyDescent="0.25">
       <c r="A170" s="5" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="B170" s="2" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
     </row>
     <row r="171" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A171" s="5" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="B171" s="2" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
     </row>
     <row r="172" spans="1:2" ht="135" x14ac:dyDescent="0.25">
       <c r="A172" s="5" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="B172" s="2" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
     </row>
     <row r="173" spans="1:2" ht="180" x14ac:dyDescent="0.25">
       <c r="A173" s="5" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="B173" s="2" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
     </row>
     <row r="174" spans="1:2" ht="180" x14ac:dyDescent="0.25">
       <c r="A174" s="5" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="B174" s="2" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
     </row>
     <row r="175" spans="1:2" ht="75" x14ac:dyDescent="0.25">
       <c r="A175" s="5" t="s">
+        <v>260</v>
+      </c>
+      <c r="B175" s="2" t="s">
         <v>261</v>
-      </c>
-      <c r="B175" s="2" t="s">
-        <v>262</v>
       </c>
     </row>
     <row r="176" spans="1:2" ht="210" x14ac:dyDescent="0.25">
       <c r="A176" s="5" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="B176" s="2" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
     </row>
     <row r="177" spans="1:2" ht="120" x14ac:dyDescent="0.25">
       <c r="A177" s="5" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="B177" s="2" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
     </row>
     <row r="178" spans="1:2" ht="105" x14ac:dyDescent="0.25">
       <c r="A178" s="5" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="B178" s="2" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
     </row>
     <row r="179" spans="1:2" ht="150" x14ac:dyDescent="0.25">
       <c r="A179" s="5" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="B179" s="2" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
     </row>
     <row r="180" spans="1:2" ht="120" x14ac:dyDescent="0.25">
       <c r="A180" s="5" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="B180" s="2" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
     </row>
     <row r="181" spans="1:2" ht="180" x14ac:dyDescent="0.25">
       <c r="A181" s="5" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="B181" s="2" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
     </row>
     <row r="182" spans="1:2" ht="120" x14ac:dyDescent="0.25">
       <c r="A182" s="5" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="B182" s="2" t="s">
-        <v>588</v>
+        <v>587</v>
       </c>
     </row>
     <row r="183" spans="1:2" ht="105" x14ac:dyDescent="0.25">
       <c r="A183" s="5" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="B183" s="2" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
     </row>
     <row r="184" spans="1:2" ht="105" x14ac:dyDescent="0.25">
       <c r="A184" s="5" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="B184" s="2" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
     </row>
     <row r="185" spans="1:2" ht="165" x14ac:dyDescent="0.25">
       <c r="A185" s="5" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="B185" s="2" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
     </row>
     <row r="186" spans="1:2" ht="60" x14ac:dyDescent="0.25">
       <c r="A186" s="5" t="s">
+        <v>432</v>
+      </c>
+      <c r="B186" s="2" t="s">
         <v>433</v>
       </c>
-      <c r="B186" s="2" t="s">
-        <v>434</v>
-      </c>
-    </row>
-    <row r="187" spans="1:2" ht="150" x14ac:dyDescent="0.25">
+    </row>
+    <row r="187" spans="1:2" ht="165" x14ac:dyDescent="0.25">
       <c r="A187" s="5" t="s">
         <v>72</v>
       </c>
       <c r="B187" s="2" t="s">
-        <v>251</v>
+        <v>595</v>
       </c>
     </row>
     <row r="188" spans="1:2" ht="180" x14ac:dyDescent="0.25">
@@ -5939,7 +5940,7 @@
         <v>77</v>
       </c>
       <c r="B191" s="2" t="s">
-        <v>572</v>
+        <v>571</v>
       </c>
     </row>
     <row r="192" spans="1:2" ht="120" x14ac:dyDescent="0.25">
@@ -5955,12 +5956,12 @@
         <v>79</v>
       </c>
       <c r="B193" s="2" t="s">
-        <v>528</v>
+        <v>527</v>
       </c>
     </row>
     <row r="194" spans="1:2" ht="60" x14ac:dyDescent="0.25">
       <c r="A194" s="5" t="s">
-        <v>527</v>
+        <v>526</v>
       </c>
       <c r="B194" s="2" t="s">
         <v>596</v>
@@ -5995,7 +5996,7 @@
         <v>98</v>
       </c>
       <c r="B198" s="2" t="s">
-        <v>477</v>
+        <v>476</v>
       </c>
     </row>
     <row r="199" spans="1:2" ht="75" x14ac:dyDescent="0.25">
@@ -6059,7 +6060,7 @@
         <v>106</v>
       </c>
       <c r="B206" s="2" t="s">
-        <v>586</v>
+        <v>585</v>
       </c>
     </row>
     <row r="207" spans="1:2" ht="45" x14ac:dyDescent="0.25">
@@ -6075,7 +6076,7 @@
         <v>115</v>
       </c>
       <c r="B208" s="2" t="s">
-        <v>587</v>
+        <v>586</v>
       </c>
     </row>
     <row r="209" spans="1:2" ht="150" x14ac:dyDescent="0.25">
@@ -6083,7 +6084,7 @@
         <v>116</v>
       </c>
       <c r="B209" s="2" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
     </row>
     <row r="210" spans="1:2" ht="255" x14ac:dyDescent="0.25">
@@ -6091,7 +6092,7 @@
         <v>117</v>
       </c>
       <c r="B210" s="2" t="s">
-        <v>508</v>
+        <v>507</v>
       </c>
     </row>
     <row r="211" spans="1:2" ht="150" x14ac:dyDescent="0.25">
@@ -6099,127 +6100,127 @@
         <v>118</v>
       </c>
       <c r="B211" s="2" t="s">
-        <v>507</v>
+        <v>506</v>
       </c>
     </row>
     <row r="212" spans="1:2" ht="285" x14ac:dyDescent="0.25">
       <c r="A212" s="5" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
       <c r="B212" s="2" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
     </row>
     <row r="213" spans="1:2" ht="180" x14ac:dyDescent="0.25">
       <c r="A213" s="5" t="s">
+        <v>446</v>
+      </c>
+      <c r="B213" s="2" t="s">
         <v>447</v>
-      </c>
-      <c r="B213" s="2" t="s">
-        <v>448</v>
       </c>
     </row>
     <row r="214" spans="1:2" ht="105" x14ac:dyDescent="0.25">
       <c r="A214" s="5" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="B214" s="2" t="s">
-        <v>455</v>
+        <v>454</v>
       </c>
     </row>
     <row r="215" spans="1:2" ht="165" x14ac:dyDescent="0.25">
       <c r="A215" s="5" t="s">
-        <v>450</v>
+        <v>449</v>
       </c>
       <c r="B215" s="2" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
     </row>
     <row r="216" spans="1:2" ht="135" x14ac:dyDescent="0.25">
       <c r="A216" s="5" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
       <c r="B216" s="2" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
     </row>
     <row r="217" spans="1:2" ht="120" x14ac:dyDescent="0.25">
       <c r="A217" s="5" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="B217" s="2" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
     </row>
     <row r="218" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A218" s="5" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="B218" s="2" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
     </row>
     <row r="219" spans="1:2" ht="75" x14ac:dyDescent="0.25">
       <c r="A219" s="5" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
       <c r="B219" s="2" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
     </row>
     <row r="220" spans="1:2" ht="75" x14ac:dyDescent="0.25">
       <c r="A220" s="5" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="B220" s="2" t="s">
-        <v>505</v>
+        <v>504</v>
       </c>
     </row>
     <row r="221" spans="1:2" ht="165" x14ac:dyDescent="0.25">
       <c r="A221" s="5" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="B221" s="2" t="s">
-        <v>504</v>
+        <v>503</v>
       </c>
     </row>
     <row r="222" spans="1:2" ht="180" x14ac:dyDescent="0.25">
       <c r="A222" s="5" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
       <c r="B222" s="2" t="s">
-        <v>503</v>
+        <v>502</v>
       </c>
     </row>
     <row r="223" spans="1:2" ht="45" x14ac:dyDescent="0.25">
       <c r="A223" s="5" t="s">
+        <v>464</v>
+      </c>
+      <c r="B223" s="2" t="s">
         <v>465</v>
-      </c>
-      <c r="B223" s="2" t="s">
-        <v>466</v>
       </c>
     </row>
     <row r="224" spans="1:2" ht="60" x14ac:dyDescent="0.25">
       <c r="A224" s="5" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="B224" s="2" t="s">
-        <v>472</v>
+        <v>471</v>
       </c>
     </row>
     <row r="225" spans="1:2" ht="180" x14ac:dyDescent="0.25">
       <c r="A225" s="5" t="s">
-        <v>470</v>
+        <v>469</v>
       </c>
       <c r="B225" s="2" t="s">
-        <v>474</v>
+        <v>473</v>
       </c>
     </row>
     <row r="226" spans="1:2" ht="60" x14ac:dyDescent="0.25">
       <c r="A226" s="5" t="s">
-        <v>471</v>
+        <v>470</v>
       </c>
       <c r="B226" s="2" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
     </row>
     <row r="227" spans="1:2" ht="117.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -6235,7 +6236,7 @@
         <v>31</v>
       </c>
       <c r="B228" s="2" t="s">
-        <v>456</v>
+        <v>455</v>
       </c>
     </row>
     <row r="229" spans="1:2" ht="45" x14ac:dyDescent="0.25">
@@ -6331,7 +6332,7 @@
         <v>67</v>
       </c>
       <c r="B240" s="2" t="s">
-        <v>499</v>
+        <v>498</v>
       </c>
     </row>
     <row r="241" spans="1:2" ht="165" x14ac:dyDescent="0.25">
@@ -6355,7 +6356,7 @@
         <v>11</v>
       </c>
       <c r="B243" s="2" t="s">
-        <v>479</v>
+        <v>478</v>
       </c>
     </row>
     <row r="244" spans="1:2" ht="180" x14ac:dyDescent="0.25">
@@ -6395,7 +6396,7 @@
         <v>5</v>
       </c>
       <c r="B248" s="2" t="s">
-        <v>565</v>
+        <v>564</v>
       </c>
     </row>
     <row r="249" spans="1:2" ht="150" x14ac:dyDescent="0.25">
@@ -6403,7 +6404,7 @@
         <v>6</v>
       </c>
       <c r="B249" s="2" t="s">
-        <v>567</v>
+        <v>566</v>
       </c>
     </row>
     <row r="250" spans="1:2" ht="255" x14ac:dyDescent="0.25">
@@ -6411,7 +6412,7 @@
         <v>7</v>
       </c>
       <c r="B250" s="2" t="s">
-        <v>595</v>
+        <v>594</v>
       </c>
     </row>
     <row r="251" spans="1:2" ht="78.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -6419,7 +6420,7 @@
         <v>8</v>
       </c>
       <c r="B251" s="2" t="s">
-        <v>566</v>
+        <v>565</v>
       </c>
     </row>
     <row r="252" spans="1:2" ht="104.65" customHeight="1" x14ac:dyDescent="0.25">
@@ -6507,7 +6508,7 @@
         <v>149</v>
       </c>
       <c r="B262" s="3" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
     </row>
     <row r="263" spans="1:2" ht="60" x14ac:dyDescent="0.25">
@@ -6523,7 +6524,7 @@
         <v>156</v>
       </c>
       <c r="B264" s="3" t="s">
-        <v>510</v>
+        <v>509</v>
       </c>
     </row>
     <row r="265" spans="1:2" ht="165" x14ac:dyDescent="0.25">
@@ -6531,7 +6532,7 @@
         <v>159</v>
       </c>
       <c r="B265" s="3" t="s">
-        <v>509</v>
+        <v>508</v>
       </c>
     </row>
     <row r="266" spans="1:2" ht="165" x14ac:dyDescent="0.25">
@@ -6539,31 +6540,31 @@
         <v>157</v>
       </c>
       <c r="B266" s="3" t="s">
-        <v>490</v>
+        <v>489</v>
       </c>
     </row>
     <row r="267" spans="1:2" ht="195" x14ac:dyDescent="0.25">
       <c r="A267" s="1" t="s">
-        <v>487</v>
+        <v>486</v>
       </c>
       <c r="B267" s="3" t="s">
-        <v>492</v>
+        <v>491</v>
       </c>
     </row>
     <row r="268" spans="1:2" ht="135" x14ac:dyDescent="0.25">
       <c r="A268" s="1" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="B268" s="3" t="s">
-        <v>593</v>
+        <v>592</v>
       </c>
     </row>
     <row r="269" spans="1:2" ht="150" x14ac:dyDescent="0.25">
       <c r="A269" s="1" t="s">
-        <v>489</v>
+        <v>488</v>
       </c>
       <c r="B269" s="3" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
     </row>
     <row r="270" spans="1:2" ht="75" x14ac:dyDescent="0.25">
@@ -6624,127 +6625,127 @@
     </row>
     <row r="277" spans="1:2" ht="165" x14ac:dyDescent="0.25">
       <c r="A277" s="1" t="s">
-        <v>481</v>
+        <v>480</v>
       </c>
       <c r="B277" s="3" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
     </row>
     <row r="278" spans="1:2" ht="105" x14ac:dyDescent="0.25">
       <c r="A278" s="1" t="s">
-        <v>482</v>
+        <v>481</v>
       </c>
       <c r="B278" s="3" t="s">
-        <v>484</v>
+        <v>483</v>
       </c>
     </row>
     <row r="279" spans="1:2" ht="210" x14ac:dyDescent="0.25">
       <c r="A279" s="1" t="s">
-        <v>483</v>
+        <v>482</v>
       </c>
       <c r="B279" s="3" t="s">
-        <v>592</v>
+        <v>591</v>
       </c>
     </row>
     <row r="280" spans="1:2" ht="120" x14ac:dyDescent="0.25">
       <c r="A280" s="1" t="s">
-        <v>485</v>
+        <v>484</v>
       </c>
       <c r="B280" s="3" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
     </row>
     <row r="281" spans="1:2" ht="105" x14ac:dyDescent="0.25">
       <c r="A281" s="1" t="s">
-        <v>486</v>
+        <v>485</v>
       </c>
       <c r="B281" s="3" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
     </row>
     <row r="282" spans="1:2" ht="270" x14ac:dyDescent="0.25">
       <c r="A282" s="1" t="s">
-        <v>540</v>
+        <v>539</v>
       </c>
       <c r="B282" s="3" t="s">
-        <v>555</v>
+        <v>554</v>
       </c>
     </row>
     <row r="283" spans="1:2" ht="150" x14ac:dyDescent="0.25">
       <c r="A283" s="1" t="s">
-        <v>541</v>
+        <v>540</v>
       </c>
       <c r="B283" s="3" t="s">
-        <v>550</v>
+        <v>549</v>
       </c>
     </row>
     <row r="284" spans="1:2" ht="60" x14ac:dyDescent="0.25">
       <c r="A284" s="1" t="s">
-        <v>542</v>
+        <v>541</v>
       </c>
       <c r="B284" s="3" t="s">
-        <v>556</v>
+        <v>555</v>
       </c>
     </row>
     <row r="285" spans="1:2" ht="60" x14ac:dyDescent="0.25">
       <c r="A285" s="1" t="s">
-        <v>543</v>
+        <v>542</v>
       </c>
       <c r="B285" s="3" t="s">
-        <v>551</v>
+        <v>550</v>
       </c>
     </row>
     <row r="286" spans="1:2" ht="60" x14ac:dyDescent="0.25">
       <c r="A286" s="1" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
       <c r="B286" s="3" t="s">
-        <v>553</v>
+        <v>552</v>
       </c>
     </row>
     <row r="287" spans="1:2" ht="60" x14ac:dyDescent="0.25">
       <c r="A287" s="1" t="s">
-        <v>545</v>
+        <v>544</v>
       </c>
       <c r="B287" s="3" t="s">
-        <v>552</v>
+        <v>551</v>
       </c>
     </row>
     <row r="288" spans="1:2" ht="60" x14ac:dyDescent="0.25">
       <c r="A288" s="1" t="s">
-        <v>546</v>
+        <v>545</v>
       </c>
       <c r="B288" s="3" t="s">
-        <v>554</v>
+        <v>553</v>
       </c>
     </row>
     <row r="289" spans="1:2" ht="60" x14ac:dyDescent="0.25">
       <c r="A289" s="1" t="s">
-        <v>547</v>
+        <v>546</v>
       </c>
       <c r="B289" s="3" t="s">
-        <v>557</v>
+        <v>556</v>
       </c>
     </row>
     <row r="290" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A290" s="1" t="s">
-        <v>548</v>
+        <v>547</v>
       </c>
       <c r="B290" s="3" t="s">
-        <v>558</v>
+        <v>557</v>
       </c>
     </row>
     <row r="291" spans="1:2" ht="195" x14ac:dyDescent="0.25">
       <c r="A291" s="1" t="s">
-        <v>549</v>
+        <v>548</v>
       </c>
       <c r="B291" s="3" t="s">
-        <v>559</v>
+        <v>558</v>
       </c>
     </row>
     <row r="292" spans="1:2" ht="180" x14ac:dyDescent="0.25">
       <c r="A292" s="1" t="s">
-        <v>493</v>
+        <v>492</v>
       </c>
       <c r="B292" s="3" t="s">
         <v>597</v>
@@ -6752,58 +6753,58 @@
     </row>
     <row r="293" spans="1:2" ht="120" x14ac:dyDescent="0.25">
       <c r="A293" s="1" t="s">
-        <v>494</v>
+        <v>493</v>
       </c>
       <c r="B293" s="3" t="s">
-        <v>577</v>
+        <v>576</v>
       </c>
     </row>
     <row r="294" spans="1:2" ht="135" x14ac:dyDescent="0.25">
       <c r="A294" s="1" t="s">
-        <v>495</v>
+        <v>494</v>
       </c>
       <c r="B294" s="3" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
     </row>
     <row r="295" spans="1:2" ht="210" x14ac:dyDescent="0.25">
       <c r="A295" s="1" t="s">
+        <v>530</v>
+      </c>
+      <c r="B295" s="3" t="s">
         <v>531</v>
-      </c>
-      <c r="B295" s="3" t="s">
-        <v>532</v>
       </c>
     </row>
     <row r="296" spans="1:2" ht="45" x14ac:dyDescent="0.25">
       <c r="A296" s="1" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="B296" s="3" t="s">
-        <v>537</v>
+        <v>536</v>
       </c>
     </row>
     <row r="297" spans="1:2" ht="45" x14ac:dyDescent="0.25">
       <c r="A297" s="1" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="B297" s="3" t="s">
-        <v>538</v>
+        <v>537</v>
       </c>
     </row>
     <row r="298" spans="1:2" ht="135" x14ac:dyDescent="0.25">
       <c r="A298" s="1" t="s">
-        <v>535</v>
+        <v>534</v>
       </c>
       <c r="B298" s="3" t="s">
-        <v>539</v>
+        <v>538</v>
       </c>
     </row>
     <row r="299" spans="1:2" ht="75" x14ac:dyDescent="0.25">
       <c r="A299" s="1" t="s">
-        <v>536</v>
+        <v>535</v>
       </c>
       <c r="B299" s="3" t="s">
-        <v>560</v>
+        <v>559</v>
       </c>
     </row>
     <row r="303" spans="1:2" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Specified that MG is nto optional for MG fire
</commit_message>
<xml_diff>
--- a/DesignDocs/Rules.xlsx
+++ b/DesignDocs/Rules.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cstew\source\repos\PattonsBest\DesignDocs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{9F78F578-95E3-4BE6-9A0E-7206975CEEF2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{B18B1163-1D42-46C5-86B9-96809C340600}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{89590866-6083-4176-8CBF-8C95C9BA24C2}"/>
   </bookViews>
@@ -4006,6 +4006,29 @@
 If you retreat from the Battle Board, go to &lt;InlineUIContainer&gt;&lt;Button Content='r20.45' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;</t>
   </si>
   <si>
+    <t>&lt;Bold&gt;r29.0 Fuel (Optional)&lt;/Bold&gt;
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+Only optional if not using digital game.
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+All Sherman tank models carry a maxium of 35 units of fuel, where each unit equals 5 gallons (175 gallons total). During the Time Check step 
+&lt;InlineUIContainer&gt;&lt;Button Content='r4.3' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; of the sequence of play, when you determine the amount of time and ammo already expended for the day, 
+the number rolled also deteremines the number of fuel units already used.
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+Subtract the number rolled from 35 to determine the number of fuel units remaining. 
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+Thereafter, fuel is consumed for action on both the Movement and Battle Boards, and is subtracted from the remaining total with each use. 
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+&lt;InlineUIContainer&gt;&lt;Button Content='r29.1' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; Movement Board Fuel Use&lt;LineBreak/&gt;
+&lt;InlineUIContainer&gt;&lt;Button Content='r29.2' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; Battle Board Fuel Use</t>
+  </si>
+  <si>
+    <t>&lt;Bold&gt;r16.3 Machine Gun (MG) Ammo (Optional)&lt;/Bold&gt; 
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+Only optional if not using digital game.
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+All rules dealing with MG ammunition should be considered optional and be followed only by choice. For most players, the additional problems posed by the consideration of MG ammo are not worth the record keeping involved. Continue to check for MG malfunctions, but otherwise assume there is sufficient MG ammo on hand for all firing.</t>
+  </si>
+  <si>
     <t>&lt;Bold&gt;r16.0 Ammunition (Ammo)&lt;/Bold&gt; 
 &lt;LineBreak/&gt;&lt;LineBreak/&gt;
 Ammo is loaded into your tank at the beginning of each scenerio as part of morning briefing 
@@ -4016,26 +4039,7 @@
 &lt;InlineUIContainer&gt;&lt;Button Content='r16.0a' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; Details&lt;LineBreak/&gt;
 &lt;InlineUIContainer&gt;&lt;Button Content='r16.1' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;  Ammo Types&lt;LineBreak/&gt;
 &lt;InlineUIContainer&gt;&lt;Button Content='r16.2' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;  Loading Ammo&lt;LineBreak/&gt;
-&lt;InlineUIContainer&gt;&lt;Button Content='r16.3' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; Machine Gun (MG) Ammo (Only Optional if not Using Digital Game)</t>
-  </si>
-  <si>
-    <t>&lt;Bold&gt;r16.3 Machine Gun (MG) Ammo (Only Optional if not Using Digital Game)&lt;/Bold&gt; 
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-All rules dealing with MG ammunition should be considered optional and be followed only by choice. For most players, the additional problems posed by the consideration of MG ammo are not worth the record keeping involved. Continue to check for MG malfunctions, but otherwise assume there is sufficient MG ammo on hand for all firing.</t>
-  </si>
-  <si>
-    <t>&lt;Bold&gt;r29.0 Fuel (Only Optional if not Using Digital Game)&lt;/Bold&gt;
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-All Sherman tank models carry a maxium of 35 units of fuel, where each unit equals 5 gallons (175 gallons total). During the Time Check step 
-&lt;InlineUIContainer&gt;&lt;Button Content='r4.3' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; of the sequence of play, when you determine the amount of time and ammo already expended for the day, 
-the number rolled also deteremines the number of fuel units already used.
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-Subtract the number rolled from 35 to determine the number of fuel units remaining. 
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-Thereafter, fuel is consumed for action on both the Movement and Battle Boards, and is subtracted from the remaining total with each use. 
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-&lt;InlineUIContainer&gt;&lt;Button Content='r29.1' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; Movement Board Fuel Use&lt;LineBreak/&gt;
-&lt;InlineUIContainer&gt;&lt;Button Content='r29.2' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; Battle Board Fuel Use</t>
+&lt;InlineUIContainer&gt;&lt;Button Content='r16.3' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;  Machine Gun (MG) Ammo</t>
   </si>
 </sst>
 </file>
@@ -5908,7 +5912,7 @@
         <v>72</v>
       </c>
       <c r="B187" s="2" t="s">
-        <v>595</v>
+        <v>597</v>
       </c>
     </row>
     <row r="188" spans="1:2" ht="180" x14ac:dyDescent="0.25">
@@ -5959,7 +5963,7 @@
         <v>527</v>
       </c>
     </row>
-    <row r="194" spans="1:2" ht="60" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A194" s="5" t="s">
         <v>526</v>
       </c>
@@ -6743,12 +6747,12 @@
         <v>558</v>
       </c>
     </row>
-    <row r="292" spans="1:2" ht="180" x14ac:dyDescent="0.25">
+    <row r="292" spans="1:2" ht="210" x14ac:dyDescent="0.25">
       <c r="A292" s="1" t="s">
         <v>492</v>
       </c>
       <c r="B292" s="3" t="s">
-        <v>597</v>
+        <v>595</v>
       </c>
     </row>
     <row r="293" spans="1:2" ht="120" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Add clarity to MG fire use
</commit_message>
<xml_diff>
--- a/DesignDocs/Rules.xlsx
+++ b/DesignDocs/Rules.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cstew\source\repos\PattonsBest\DesignDocs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B18B1163-1D42-46C5-86B9-96809C340600}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{1C16DA48-99D3-412E-93B5-A1F62CF8D8EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{89590866-6083-4176-8CBF-8C95C9BA24C2}"/>
   </bookViews>
@@ -4022,13 +4022,6 @@
 &lt;InlineUIContainer&gt;&lt;Button Content='r29.2' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; Battle Board Fuel Use</t>
   </si>
   <si>
-    <t>&lt;Bold&gt;r16.3 Machine Gun (MG) Ammo (Optional)&lt;/Bold&gt; 
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-Only optional if not using digital game.
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-All rules dealing with MG ammunition should be considered optional and be followed only by choice. For most players, the additional problems posed by the consideration of MG ammo are not worth the record keeping involved. Continue to check for MG malfunctions, but otherwise assume there is sufficient MG ammo on hand for all firing.</t>
-  </si>
-  <si>
     <t>&lt;Bold&gt;r16.0 Ammunition (Ammo)&lt;/Bold&gt; 
 &lt;LineBreak/&gt;&lt;LineBreak/&gt;
 Ammo is loaded into your tank at the beginning of each scenerio as part of morning briefing 
@@ -4040,6 +4033,15 @@
 &lt;InlineUIContainer&gt;&lt;Button Content='r16.1' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;  Ammo Types&lt;LineBreak/&gt;
 &lt;InlineUIContainer&gt;&lt;Button Content='r16.2' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;  Loading Ammo&lt;LineBreak/&gt;
 &lt;InlineUIContainer&gt;&lt;Button Content='r16.3' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;  Machine Gun (MG) Ammo</t>
+  </si>
+  <si>
+    <t>&lt;Bold&gt;r16.3 Machine Gun (MG) Ammo (Optional)&lt;/Bold&gt; 
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+Only optional if not using digital game.
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+All rules dealing with MG ammunition should be considered optional and be followed only by choice. For most players, the additional problems posed by the consideration of MG ammo are not worth the record keeping involved. Continue to check for MG malfunctions, but otherwise assume there is sufficient MG ammo on hand for all firing.
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+See &lt;InlineUIContainer&gt;&lt;Button Content='r22.21' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; for machine gun ammo use.</t>
   </si>
 </sst>
 </file>
@@ -5912,7 +5914,7 @@
         <v>72</v>
       </c>
       <c r="B187" s="2" t="s">
-        <v>597</v>
+        <v>596</v>
       </c>
     </row>
     <row r="188" spans="1:2" ht="180" x14ac:dyDescent="0.25">
@@ -5963,12 +5965,12 @@
         <v>527</v>
       </c>
     </row>
-    <row r="194" spans="1:2" ht="90" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:2" ht="120" x14ac:dyDescent="0.25">
       <c r="A194" s="5" t="s">
         <v>526</v>
       </c>
       <c r="B194" s="2" t="s">
-        <v>596</v>
+        <v>597</v>
       </c>
     </row>
     <row r="195" spans="1:2" ht="240" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Fix mispelling on Advance Fire rule r22.13
</commit_message>
<xml_diff>
--- a/DesignDocs/Rules.xlsx
+++ b/DesignDocs/Rules.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cstew\source\repos\PattonsBest\DesignDocs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{81B90228-6087-4022-BB23-B7831271B390}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{4D47EE94-4DB6-4CE2-B833-606E790A590F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{89590866-6083-4176-8CBF-8C95C9BA24C2}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{89590866-6083-4176-8CBF-8C95C9BA24C2}"/>
   </bookViews>
   <sheets>
     <sheet name="Rules" sheetId="1" r:id="rId1"/>
@@ -871,20 +871,6 @@
 &lt;InlineUIContainer&gt;&lt;Button Content='AAR' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;.</t>
   </si>
   <si>
-    <t>&lt;Bold&gt;r22.13 Advancing Fire Resolution&lt;/Bold&gt;
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-Advancing Fire is resolved in each Battle Board zone containing both an Advance Fire marker and enemy units during Battle Step 
-&lt;InlineUIContainer&gt;&lt;Button Content='r4.64' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;. 
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-For each, roll on the 
-&lt;InlineUIContainer&gt;&lt;Button Content='Friendly Action' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; 
-Table against each unit in the zone. 
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-Enemy units kocked out are considered to be withdrawing and are not destroyed. No victory points are awarded. 
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-Remove the Advancing Fire markers from the Battle Board after resolving.</t>
-  </si>
-  <si>
     <t>r23.0</t>
   </si>
   <si>
@@ -4042,6 +4028,20 @@
 All rules dealing with MG ammunition should be considered optional and be followed only by choice. For most players, the additional problems posed by the consideration of MG ammo are not worth the record keeping involved. Continue to check for MG malfunctions, but otherwise assume there is sufficient MG ammo on hand for all firing.
 &lt;LineBreak/&gt;&lt;LineBreak/&gt;
 See &lt;InlineUIContainer&gt;&lt;Button Content='r22.11' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; for machine gun ammo use.</t>
+  </si>
+  <si>
+    <t>&lt;Bold&gt;r22.13 Advancing Fire Resolution&lt;/Bold&gt;
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+Advancing Fire is resolved in each Battle Board zone containing both an Advance Fire marker and enemy units during Battle Step 
+&lt;InlineUIContainer&gt;&lt;Button Content='r4.64' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;. 
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+For each, roll on the 
+&lt;InlineUIContainer&gt;&lt;Button Content='Friendly Action' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; 
+Table against each unit in the zone. 
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+Enemy units knocked out are considered to be withdrawing and are not destroyed. No victory points are awarded. 
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+Remove the Advancing Fire markers from the Battle Board after resolving.</t>
   </si>
 </sst>
 </file>
@@ -4426,7 +4426,7 @@
         <v>46</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>568</v>
+        <v>567</v>
       </c>
     </row>
     <row r="2" spans="1:2" ht="91.7" customHeight="1" x14ac:dyDescent="0.25">
@@ -4458,7 +4458,7 @@
         <v>17</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>569</v>
+        <v>568</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="120" x14ac:dyDescent="0.25">
@@ -4466,7 +4466,7 @@
         <v>18</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="45" x14ac:dyDescent="0.25">
@@ -4498,7 +4498,7 @@
         <v>49</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
     </row>
     <row r="11" spans="1:2" ht="165" x14ac:dyDescent="0.25">
@@ -4538,7 +4538,7 @@
         <v>85</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
     </row>
     <row r="16" spans="1:2" ht="120" x14ac:dyDescent="0.25">
@@ -4570,7 +4570,7 @@
         <v>89</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>593</v>
+        <v>592</v>
       </c>
     </row>
     <row r="20" spans="1:2" ht="120" x14ac:dyDescent="0.25">
@@ -4602,7 +4602,7 @@
         <v>125</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
     </row>
     <row r="24" spans="1:2" ht="120" x14ac:dyDescent="0.25">
@@ -4610,7 +4610,7 @@
         <v>126</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="25" spans="1:2" ht="135" x14ac:dyDescent="0.25">
@@ -4618,7 +4618,7 @@
         <v>127</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="26" spans="1:2" ht="210" x14ac:dyDescent="0.25">
@@ -4642,7 +4642,7 @@
         <v>130</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
     </row>
     <row r="29" spans="1:2" ht="150" x14ac:dyDescent="0.25">
@@ -4650,7 +4650,7 @@
         <v>131</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>495</v>
+        <v>494</v>
       </c>
     </row>
     <row r="30" spans="1:2" ht="120" x14ac:dyDescent="0.25">
@@ -4658,7 +4658,7 @@
         <v>132</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>497</v>
+        <v>496</v>
       </c>
     </row>
     <row r="31" spans="1:2" ht="360" x14ac:dyDescent="0.25">
@@ -4666,359 +4666,359 @@
         <v>133</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="32" spans="1:2" ht="135" x14ac:dyDescent="0.25">
       <c r="A32" s="5" t="s">
+        <v>219</v>
+      </c>
+      <c r="B32" s="2" t="s">
         <v>220</v>
-      </c>
-      <c r="B32" s="2" t="s">
-        <v>221</v>
       </c>
     </row>
     <row r="33" spans="1:2" ht="60" x14ac:dyDescent="0.25">
       <c r="A33" s="5" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>499</v>
+        <v>498</v>
       </c>
     </row>
     <row r="34" spans="1:2" ht="165" x14ac:dyDescent="0.25">
       <c r="A34" s="5" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
     </row>
     <row r="35" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A35" s="5" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
     </row>
     <row r="36" spans="1:2" ht="105" x14ac:dyDescent="0.25">
       <c r="A36" s="5" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="37" spans="1:2" ht="285" x14ac:dyDescent="0.25">
       <c r="A37" s="5" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>500</v>
+        <v>499</v>
       </c>
     </row>
     <row r="38" spans="1:2" ht="135" x14ac:dyDescent="0.25">
       <c r="A38" s="5" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
     </row>
     <row r="39" spans="1:2" ht="75" x14ac:dyDescent="0.25">
       <c r="A39" s="5" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>474</v>
+        <v>473</v>
       </c>
     </row>
     <row r="40" spans="1:2" ht="150" x14ac:dyDescent="0.25">
       <c r="A40" s="5" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
     </row>
     <row r="41" spans="1:2" ht="150" x14ac:dyDescent="0.25">
       <c r="A41" s="5" t="s">
-        <v>439</v>
+        <v>438</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>479</v>
+        <v>478</v>
       </c>
     </row>
     <row r="42" spans="1:2" ht="135" x14ac:dyDescent="0.25">
       <c r="A42" s="5" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>524</v>
+        <v>523</v>
       </c>
     </row>
     <row r="43" spans="1:2" ht="105" x14ac:dyDescent="0.25">
       <c r="A43" s="5" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
     </row>
     <row r="44" spans="1:2" ht="285" x14ac:dyDescent="0.25">
       <c r="A44" s="5" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>529</v>
+        <v>528</v>
       </c>
     </row>
     <row r="45" spans="1:2" ht="135" x14ac:dyDescent="0.25">
       <c r="A45" s="5" t="s">
-        <v>521</v>
+        <v>520</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>528</v>
+        <v>527</v>
       </c>
     </row>
     <row r="46" spans="1:2" ht="210" x14ac:dyDescent="0.25">
       <c r="A46" s="5" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
     </row>
     <row r="47" spans="1:2" ht="300" x14ac:dyDescent="0.25">
       <c r="A47" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="B47" s="2" t="s">
-        <v>501</v>
+        <v>500</v>
       </c>
     </row>
     <row r="48" spans="1:2" ht="150" x14ac:dyDescent="0.25">
       <c r="A48" s="5" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>510</v>
+        <v>509</v>
       </c>
     </row>
     <row r="49" spans="1:2" ht="180" x14ac:dyDescent="0.25">
       <c r="A49" s="5" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="B49" s="2" t="s">
-        <v>511</v>
+        <v>510</v>
       </c>
     </row>
     <row r="50" spans="1:2" ht="60" x14ac:dyDescent="0.25">
       <c r="A50" s="5" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
       <c r="B50" s="2" t="s">
-        <v>515</v>
+        <v>514</v>
       </c>
     </row>
     <row r="51" spans="1:2" ht="240" x14ac:dyDescent="0.25">
       <c r="A51" s="5" t="s">
-        <v>512</v>
+        <v>511</v>
       </c>
       <c r="B51" s="2" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
     </row>
     <row r="52" spans="1:2" ht="390" x14ac:dyDescent="0.25">
       <c r="A52" s="5" t="s">
-        <v>514</v>
+        <v>513</v>
       </c>
       <c r="B52" s="2" t="s">
-        <v>516</v>
+        <v>515</v>
       </c>
     </row>
     <row r="53" spans="1:2" ht="195" x14ac:dyDescent="0.25">
       <c r="A53" s="5" t="s">
-        <v>513</v>
+        <v>512</v>
       </c>
       <c r="B53" s="2" t="s">
-        <v>517</v>
+        <v>516</v>
       </c>
     </row>
     <row r="54" spans="1:2" ht="105" x14ac:dyDescent="0.25">
       <c r="A54" s="5" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="B54" s="2" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
     </row>
     <row r="55" spans="1:2" ht="135" x14ac:dyDescent="0.25">
       <c r="A55" s="5" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="B55" s="2" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
     </row>
     <row r="56" spans="1:2" ht="135" x14ac:dyDescent="0.25">
       <c r="A56" s="5" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="B56" s="2" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
     </row>
     <row r="57" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A57" s="5" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="B57" s="2" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
     </row>
     <row r="58" spans="1:2" ht="105" x14ac:dyDescent="0.25">
       <c r="A58" s="5" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="B58" s="2" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
     </row>
     <row r="59" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A59" s="5" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="B59" s="2" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
     </row>
     <row r="60" spans="1:2" ht="135" x14ac:dyDescent="0.25">
       <c r="A60" s="5" t="s">
+        <v>196</v>
+      </c>
+      <c r="B60" s="2" t="s">
         <v>197</v>
-      </c>
-      <c r="B60" s="2" t="s">
-        <v>198</v>
       </c>
     </row>
     <row r="61" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A61" s="5" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="B61" s="2" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
     </row>
     <row r="62" spans="1:2" ht="120" x14ac:dyDescent="0.25">
       <c r="A62" s="5" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="B62" s="2" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
     </row>
     <row r="63" spans="1:2" ht="180" x14ac:dyDescent="0.25">
       <c r="A63" s="5" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="B63" s="2" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
     </row>
     <row r="64" spans="1:2" ht="165" x14ac:dyDescent="0.25">
       <c r="A64" s="5" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="B64" s="2" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
     </row>
     <row r="65" spans="1:2" ht="135" x14ac:dyDescent="0.25">
       <c r="A65" s="5" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="B65" s="2" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
     </row>
     <row r="66" spans="1:2" ht="180" x14ac:dyDescent="0.25">
       <c r="A66" s="5" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="B66" s="2" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
     </row>
     <row r="67" spans="1:2" ht="75" x14ac:dyDescent="0.25">
       <c r="A67" s="5" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="B67" s="2" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
     </row>
     <row r="68" spans="1:2" ht="195" x14ac:dyDescent="0.25">
       <c r="A68" s="5" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B68" s="2" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
     </row>
     <row r="69" spans="1:2" ht="135" x14ac:dyDescent="0.25">
       <c r="A69" s="5" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="B69" s="2" t="s">
-        <v>505</v>
+        <v>504</v>
       </c>
     </row>
     <row r="70" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A70" s="5" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B70" s="2" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
     </row>
     <row r="71" spans="1:2" ht="150" x14ac:dyDescent="0.25">
       <c r="A71" s="5" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="B71" s="2" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
     </row>
     <row r="72" spans="1:2" ht="135" x14ac:dyDescent="0.25">
       <c r="A72" s="5" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="B72" s="2" t="s">
-        <v>582</v>
+        <v>581</v>
       </c>
     </row>
     <row r="73" spans="1:2" ht="195" x14ac:dyDescent="0.25">
       <c r="A73" s="5" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="B73" s="2" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
     </row>
     <row r="74" spans="1:2" ht="120" x14ac:dyDescent="0.25">
       <c r="A74" s="5" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="B74" s="2" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
     </row>
     <row r="75" spans="1:2" ht="105" x14ac:dyDescent="0.25">
       <c r="A75" s="5" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="B75" s="2" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="76" spans="1:2" ht="136.15" customHeight="1" x14ac:dyDescent="0.25">
@@ -5047,866 +5047,866 @@
     </row>
     <row r="79" spans="1:2" ht="165" x14ac:dyDescent="0.25">
       <c r="A79" s="5" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="B79" s="2" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
     </row>
     <row r="80" spans="1:2" ht="135" x14ac:dyDescent="0.25">
       <c r="A80" s="5" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="B80" s="2" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
     </row>
     <row r="81" spans="1:2" ht="120" x14ac:dyDescent="0.25">
       <c r="A81" s="5" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="B81" s="2" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
     </row>
     <row r="82" spans="1:2" ht="135" x14ac:dyDescent="0.25">
       <c r="A82" s="5" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="B82" s="2" t="s">
-        <v>567</v>
+        <v>566</v>
       </c>
     </row>
     <row r="83" spans="1:2" ht="135" x14ac:dyDescent="0.25">
       <c r="A83" s="5" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="B83" s="2" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
     </row>
     <row r="84" spans="1:2" ht="75" x14ac:dyDescent="0.25">
       <c r="A84" s="5" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="B84" s="2" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
     </row>
     <row r="85" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A85" s="5" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="B85" s="2" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
     </row>
     <row r="86" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A86" s="5" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="B86" s="2" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
     </row>
     <row r="87" spans="1:2" ht="105" x14ac:dyDescent="0.25">
       <c r="A87" s="5" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="B87" s="2" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
     </row>
     <row r="88" spans="1:2" ht="135" x14ac:dyDescent="0.25">
       <c r="A88" s="5" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="B88" s="2" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
     </row>
     <row r="89" spans="1:2" ht="195" x14ac:dyDescent="0.25">
       <c r="A89" s="5" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="B89" s="2" t="s">
-        <v>581</v>
+        <v>580</v>
       </c>
     </row>
     <row r="90" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A90" s="5" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="B90" s="2" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
     </row>
     <row r="91" spans="1:2" ht="105" x14ac:dyDescent="0.25">
       <c r="A91" s="5" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="B91" s="2" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
     </row>
     <row r="92" spans="1:2" ht="105" x14ac:dyDescent="0.25">
       <c r="A92" s="5" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="B92" s="2" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
     </row>
     <row r="93" spans="1:2" ht="75" x14ac:dyDescent="0.25">
       <c r="A93" s="5" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="B93" s="2" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
     </row>
     <row r="94" spans="1:2" ht="75" x14ac:dyDescent="0.25">
       <c r="A94" s="5" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="B94" s="2" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
     </row>
     <row r="95" spans="1:2" ht="75" x14ac:dyDescent="0.25">
       <c r="A95" s="5" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="B95" s="2" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
     </row>
     <row r="96" spans="1:2" ht="150" x14ac:dyDescent="0.25">
       <c r="A96" s="5" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="B96" s="2" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
     </row>
     <row r="97" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A97" s="5" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="B97" s="2" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
     </row>
     <row r="98" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A98" s="5" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="B98" s="2" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
     </row>
     <row r="99" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A99" s="5" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="B99" s="2" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
     </row>
     <row r="100" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A100" s="5" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="B100" s="2" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="101" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A101" s="5" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="B101" s="2" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
     </row>
     <row r="102" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A102" s="5" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="B102" s="2" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
     </row>
     <row r="103" spans="1:2" ht="105" x14ac:dyDescent="0.25">
       <c r="A103" s="5" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="B103" s="2" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
     </row>
     <row r="104" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A104" s="5" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="B104" s="2" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
     </row>
     <row r="105" spans="1:2" ht="105" x14ac:dyDescent="0.25">
       <c r="A105" s="5" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="B105" s="2" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
     </row>
     <row r="106" spans="1:2" ht="120" x14ac:dyDescent="0.25">
       <c r="A106" s="5" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="B106" s="2" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
     </row>
     <row r="107" spans="1:2" ht="105" x14ac:dyDescent="0.25">
       <c r="A107" s="5" t="s">
+        <v>289</v>
+      </c>
+      <c r="B107" s="2" t="s">
         <v>290</v>
-      </c>
-      <c r="B107" s="2" t="s">
-        <v>291</v>
       </c>
     </row>
     <row r="108" spans="1:2" ht="135" x14ac:dyDescent="0.25">
       <c r="A108" s="5" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="B108" s="2" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
     </row>
     <row r="109" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A109" s="5" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="B109" s="2" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
     </row>
     <row r="110" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A110" s="5" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="B110" s="2" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
     </row>
     <row r="111" spans="1:2" ht="75" x14ac:dyDescent="0.25">
       <c r="A111" s="5" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="B111" s="2" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
     </row>
     <row r="112" spans="1:2" ht="105" x14ac:dyDescent="0.25">
       <c r="A112" s="5" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="B112" s="2" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
     </row>
     <row r="113" spans="1:2" ht="255" x14ac:dyDescent="0.25">
       <c r="A113" s="5" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="B113" s="2" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
     </row>
     <row r="114" spans="1:2" ht="210" x14ac:dyDescent="0.25">
       <c r="A114" s="5" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="B114" s="2" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
     </row>
     <row r="115" spans="1:2" ht="135" x14ac:dyDescent="0.25">
       <c r="A115" s="5" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="B115" s="2" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
     </row>
     <row r="116" spans="1:2" ht="105" x14ac:dyDescent="0.25">
       <c r="A116" s="5" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="B116" s="2" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
     </row>
     <row r="117" spans="1:2" ht="120" x14ac:dyDescent="0.25">
       <c r="A117" s="5" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="B117" s="2" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
     </row>
     <row r="118" spans="1:2" ht="60" x14ac:dyDescent="0.25">
       <c r="A118" s="5" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="B118" s="2" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
     </row>
     <row r="119" spans="1:2" ht="135" x14ac:dyDescent="0.25">
       <c r="A119" s="5" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="B119" s="2" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
     </row>
     <row r="120" spans="1:2" ht="75" x14ac:dyDescent="0.25">
       <c r="A120" s="5" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="B120" s="2" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
     </row>
     <row r="121" spans="1:2" ht="195" x14ac:dyDescent="0.25">
       <c r="A121" s="5" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="B121" s="2" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
     </row>
     <row r="122" spans="1:2" ht="120" x14ac:dyDescent="0.25">
       <c r="A122" s="5" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="B122" s="2" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
     </row>
     <row r="123" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A123" s="5" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="B123" s="2" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
     </row>
     <row r="124" spans="1:2" ht="45" x14ac:dyDescent="0.25">
       <c r="A124" s="5" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="B124" s="2" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
     </row>
     <row r="125" spans="1:2" ht="105" x14ac:dyDescent="0.25">
       <c r="A125" s="5" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="B125" s="2" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
     </row>
     <row r="126" spans="1:2" ht="120" x14ac:dyDescent="0.25">
       <c r="A126" s="5" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="B126" s="2" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
     </row>
     <row r="127" spans="1:2" ht="180" x14ac:dyDescent="0.25">
       <c r="A127" s="5" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="B127" s="2" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
     </row>
     <row r="128" spans="1:2" ht="180" x14ac:dyDescent="0.25">
       <c r="A128" s="5" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="B128" s="2" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
     </row>
     <row r="129" spans="1:2" ht="60" x14ac:dyDescent="0.25">
       <c r="A129" s="5" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="B129" s="2" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
     </row>
     <row r="130" spans="1:2" ht="180" x14ac:dyDescent="0.25">
       <c r="A130" s="5" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="B130" s="2" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
     </row>
     <row r="131" spans="1:2" ht="285" x14ac:dyDescent="0.25">
       <c r="A131" s="5" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="B131" s="2" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
     </row>
     <row r="132" spans="1:2" ht="60" x14ac:dyDescent="0.25">
       <c r="A132" s="5" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="B132" s="2" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
     </row>
     <row r="133" spans="1:2" ht="195" x14ac:dyDescent="0.25">
       <c r="A133" s="5" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="B133" s="2" t="s">
-        <v>573</v>
+        <v>572</v>
       </c>
     </row>
     <row r="134" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A134" s="5" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="B134" s="2" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
     </row>
     <row r="135" spans="1:2" ht="75" x14ac:dyDescent="0.25">
       <c r="A135" s="5" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="B135" s="2" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
     </row>
     <row r="136" spans="1:2" ht="135" x14ac:dyDescent="0.25">
       <c r="A136" s="5" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B136" s="2" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
     </row>
     <row r="137" spans="1:2" ht="75" x14ac:dyDescent="0.25">
       <c r="A137" s="5" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="B137" s="2" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
     </row>
     <row r="138" spans="1:2" ht="180" x14ac:dyDescent="0.25">
       <c r="A138" s="5" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="B138" s="2" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
     </row>
     <row r="139" spans="1:2" ht="255" x14ac:dyDescent="0.25">
       <c r="A139" s="5" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="B139" s="2" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
     </row>
     <row r="140" spans="1:2" ht="210" x14ac:dyDescent="0.25">
       <c r="A140" s="5" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="B140" s="2" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
     </row>
     <row r="141" spans="1:2" ht="195" x14ac:dyDescent="0.25">
       <c r="A141" s="5" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="B141" s="2" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
     </row>
     <row r="142" spans="1:2" ht="165" x14ac:dyDescent="0.25">
       <c r="A142" s="5" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="B142" s="2" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
     </row>
     <row r="143" spans="1:2" ht="108.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A143" s="5" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="B143" s="2" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
     </row>
     <row r="144" spans="1:2" ht="210" x14ac:dyDescent="0.25">
       <c r="A144" s="5" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="B144" s="2" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
     </row>
     <row r="145" spans="1:2" ht="75" x14ac:dyDescent="0.25">
       <c r="A145" s="5" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="B145" s="2" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
     </row>
     <row r="146" spans="1:2" ht="75" x14ac:dyDescent="0.25">
       <c r="A146" s="5" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="B146" s="2" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
     </row>
     <row r="147" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A147" s="5" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="B147" s="2" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
     </row>
     <row r="148" spans="1:2" ht="105" x14ac:dyDescent="0.25">
       <c r="A148" s="5" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="B148" s="2" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
     </row>
     <row r="149" spans="1:2" ht="150" x14ac:dyDescent="0.25">
       <c r="A149" s="5" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="B149" s="2" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
     </row>
     <row r="150" spans="1:2" ht="330" x14ac:dyDescent="0.25">
       <c r="A150" s="5" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="B150" s="2" t="s">
-        <v>572</v>
+        <v>571</v>
       </c>
     </row>
     <row r="151" spans="1:2" ht="195" x14ac:dyDescent="0.25">
       <c r="A151" s="5" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="B151" s="2" t="s">
-        <v>588</v>
+        <v>587</v>
       </c>
     </row>
     <row r="152" spans="1:2" ht="225" x14ac:dyDescent="0.25">
       <c r="A152" s="5" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="B152" s="2" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
     </row>
     <row r="153" spans="1:2" ht="75" x14ac:dyDescent="0.25">
       <c r="A153" s="5" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="B153" s="2" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
     </row>
     <row r="154" spans="1:2" ht="75" x14ac:dyDescent="0.25">
       <c r="A154" s="5" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="B154" s="2" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
     </row>
     <row r="155" spans="1:2" ht="75" x14ac:dyDescent="0.25">
       <c r="A155" s="5" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="B155" s="2" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
     </row>
     <row r="156" spans="1:2" ht="75" x14ac:dyDescent="0.25">
       <c r="A156" s="5" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="B156" s="2" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
     </row>
     <row r="157" spans="1:2" ht="75" x14ac:dyDescent="0.25">
       <c r="A157" s="5" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="B157" s="2" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
     </row>
     <row r="158" spans="1:2" ht="105" x14ac:dyDescent="0.25">
       <c r="A158" s="5" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="B158" s="2" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
     </row>
     <row r="159" spans="1:2" ht="180" x14ac:dyDescent="0.25">
       <c r="A159" s="5" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="B159" s="2" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
     </row>
     <row r="160" spans="1:2" ht="150" x14ac:dyDescent="0.25">
       <c r="A160" s="5" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="B160" s="2" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
     </row>
     <row r="161" spans="1:2" ht="60" x14ac:dyDescent="0.25">
       <c r="A161" s="5" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="B161" s="2" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
     </row>
     <row r="162" spans="1:2" ht="75" x14ac:dyDescent="0.25">
       <c r="A162" s="5" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="B162" s="2" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
     </row>
     <row r="163" spans="1:2" ht="75" x14ac:dyDescent="0.25">
       <c r="A163" s="5" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="B163" s="2" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
     </row>
     <row r="164" spans="1:2" ht="180" x14ac:dyDescent="0.25">
       <c r="A164" s="5" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="B164" s="2" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="165" spans="1:2" ht="195" x14ac:dyDescent="0.25">
       <c r="A165" s="5" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="B165" s="2" t="s">
-        <v>560</v>
+        <v>559</v>
       </c>
     </row>
     <row r="166" spans="1:2" ht="195" x14ac:dyDescent="0.25">
       <c r="A166" s="5" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="B166" s="2" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
     </row>
     <row r="167" spans="1:2" ht="75" x14ac:dyDescent="0.25">
       <c r="A167" s="5" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="B167" s="2" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
     </row>
     <row r="168" spans="1:2" ht="75" x14ac:dyDescent="0.25">
       <c r="A168" s="5" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="B168" s="2" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
     </row>
     <row r="169" spans="1:2" ht="45" x14ac:dyDescent="0.25">
       <c r="A169" s="5" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="B169" s="2" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
     </row>
     <row r="170" spans="1:2" ht="45" x14ac:dyDescent="0.25">
       <c r="A170" s="5" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="B170" s="2" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
     </row>
     <row r="171" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A171" s="5" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="B171" s="2" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
     </row>
     <row r="172" spans="1:2" ht="135" x14ac:dyDescent="0.25">
       <c r="A172" s="5" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="B172" s="2" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
     </row>
     <row r="173" spans="1:2" ht="180" x14ac:dyDescent="0.25">
       <c r="A173" s="5" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="B173" s="2" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
     </row>
     <row r="174" spans="1:2" ht="180" x14ac:dyDescent="0.25">
       <c r="A174" s="5" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="B174" s="2" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
     </row>
     <row r="175" spans="1:2" ht="75" x14ac:dyDescent="0.25">
       <c r="A175" s="5" t="s">
+        <v>259</v>
+      </c>
+      <c r="B175" s="2" t="s">
         <v>260</v>
-      </c>
-      <c r="B175" s="2" t="s">
-        <v>261</v>
       </c>
     </row>
     <row r="176" spans="1:2" ht="210" x14ac:dyDescent="0.25">
       <c r="A176" s="5" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="B176" s="2" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
     </row>
     <row r="177" spans="1:2" ht="120" x14ac:dyDescent="0.25">
       <c r="A177" s="5" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="B177" s="2" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
     </row>
     <row r="178" spans="1:2" ht="105" x14ac:dyDescent="0.25">
       <c r="A178" s="5" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="B178" s="2" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
     </row>
     <row r="179" spans="1:2" ht="150" x14ac:dyDescent="0.25">
       <c r="A179" s="5" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="B179" s="2" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
     </row>
     <row r="180" spans="1:2" ht="120" x14ac:dyDescent="0.25">
       <c r="A180" s="5" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="B180" s="2" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
     </row>
     <row r="181" spans="1:2" ht="180" x14ac:dyDescent="0.25">
       <c r="A181" s="5" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="B181" s="2" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
     </row>
     <row r="182" spans="1:2" ht="120" x14ac:dyDescent="0.25">
       <c r="A182" s="5" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="B182" s="2" t="s">
-        <v>587</v>
+        <v>586</v>
       </c>
     </row>
     <row r="183" spans="1:2" ht="105" x14ac:dyDescent="0.25">
       <c r="A183" s="5" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="B183" s="2" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
     </row>
     <row r="184" spans="1:2" ht="105" x14ac:dyDescent="0.25">
       <c r="A184" s="5" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="B184" s="2" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
     </row>
     <row r="185" spans="1:2" ht="165" x14ac:dyDescent="0.25">
       <c r="A185" s="5" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="B185" s="2" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
     </row>
     <row r="186" spans="1:2" ht="60" x14ac:dyDescent="0.25">
       <c r="A186" s="5" t="s">
+        <v>431</v>
+      </c>
+      <c r="B186" s="2" t="s">
         <v>432</v>
-      </c>
-      <c r="B186" s="2" t="s">
-        <v>433</v>
       </c>
     </row>
     <row r="187" spans="1:2" ht="165" x14ac:dyDescent="0.25">
@@ -5914,7 +5914,7 @@
         <v>72</v>
       </c>
       <c r="B187" s="2" t="s">
-        <v>596</v>
+        <v>595</v>
       </c>
     </row>
     <row r="188" spans="1:2" ht="180" x14ac:dyDescent="0.25">
@@ -5946,7 +5946,7 @@
         <v>77</v>
       </c>
       <c r="B191" s="2" t="s">
-        <v>571</v>
+        <v>570</v>
       </c>
     </row>
     <row r="192" spans="1:2" ht="120" x14ac:dyDescent="0.25">
@@ -5962,15 +5962,15 @@
         <v>79</v>
       </c>
       <c r="B193" s="2" t="s">
-        <v>527</v>
+        <v>526</v>
       </c>
     </row>
     <row r="194" spans="1:2" ht="120" x14ac:dyDescent="0.25">
       <c r="A194" s="5" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="B194" s="2" t="s">
-        <v>597</v>
+        <v>596</v>
       </c>
     </row>
     <row r="195" spans="1:2" ht="240" x14ac:dyDescent="0.25">
@@ -6002,7 +6002,7 @@
         <v>98</v>
       </c>
       <c r="B198" s="2" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
     </row>
     <row r="199" spans="1:2" ht="75" x14ac:dyDescent="0.25">
@@ -6066,7 +6066,7 @@
         <v>106</v>
       </c>
       <c r="B206" s="2" t="s">
-        <v>585</v>
+        <v>584</v>
       </c>
     </row>
     <row r="207" spans="1:2" ht="45" x14ac:dyDescent="0.25">
@@ -6082,7 +6082,7 @@
         <v>115</v>
       </c>
       <c r="B208" s="2" t="s">
-        <v>586</v>
+        <v>585</v>
       </c>
     </row>
     <row r="209" spans="1:2" ht="150" x14ac:dyDescent="0.25">
@@ -6090,7 +6090,7 @@
         <v>116</v>
       </c>
       <c r="B209" s="2" t="s">
-        <v>477</v>
+        <v>476</v>
       </c>
     </row>
     <row r="210" spans="1:2" ht="255" x14ac:dyDescent="0.25">
@@ -6098,7 +6098,7 @@
         <v>117</v>
       </c>
       <c r="B210" s="2" t="s">
-        <v>507</v>
+        <v>506</v>
       </c>
     </row>
     <row r="211" spans="1:2" ht="150" x14ac:dyDescent="0.25">
@@ -6106,127 +6106,127 @@
         <v>118</v>
       </c>
       <c r="B211" s="2" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
     </row>
     <row r="212" spans="1:2" ht="285" x14ac:dyDescent="0.25">
       <c r="A212" s="5" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="B212" s="2" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
     </row>
     <row r="213" spans="1:2" ht="180" x14ac:dyDescent="0.25">
       <c r="A213" s="5" t="s">
+        <v>445</v>
+      </c>
+      <c r="B213" s="2" t="s">
         <v>446</v>
-      </c>
-      <c r="B213" s="2" t="s">
-        <v>447</v>
       </c>
     </row>
     <row r="214" spans="1:2" ht="105" x14ac:dyDescent="0.25">
       <c r="A214" s="5" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="B214" s="2" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
     </row>
     <row r="215" spans="1:2" ht="165" x14ac:dyDescent="0.25">
       <c r="A215" s="5" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="B215" s="2" t="s">
-        <v>456</v>
+        <v>455</v>
       </c>
     </row>
     <row r="216" spans="1:2" ht="135" x14ac:dyDescent="0.25">
       <c r="A216" s="5" t="s">
-        <v>450</v>
+        <v>449</v>
       </c>
       <c r="B216" s="2" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
     </row>
     <row r="217" spans="1:2" ht="120" x14ac:dyDescent="0.25">
       <c r="A217" s="5" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
       <c r="B217" s="2" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
     </row>
     <row r="218" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A218" s="5" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="B218" s="2" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
     </row>
     <row r="219" spans="1:2" ht="75" x14ac:dyDescent="0.25">
       <c r="A219" s="5" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="B219" s="2" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
     </row>
     <row r="220" spans="1:2" ht="75" x14ac:dyDescent="0.25">
       <c r="A220" s="5" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="B220" s="2" t="s">
-        <v>504</v>
+        <v>503</v>
       </c>
     </row>
     <row r="221" spans="1:2" ht="165" x14ac:dyDescent="0.25">
       <c r="A221" s="5" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="B221" s="2" t="s">
-        <v>503</v>
+        <v>502</v>
       </c>
     </row>
     <row r="222" spans="1:2" ht="180" x14ac:dyDescent="0.25">
       <c r="A222" s="5" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="B222" s="2" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
     </row>
     <row r="223" spans="1:2" ht="45" x14ac:dyDescent="0.25">
       <c r="A223" s="5" t="s">
+        <v>463</v>
+      </c>
+      <c r="B223" s="2" t="s">
         <v>464</v>
-      </c>
-      <c r="B223" s="2" t="s">
-        <v>465</v>
       </c>
     </row>
     <row r="224" spans="1:2" ht="60" x14ac:dyDescent="0.25">
       <c r="A224" s="5" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="B224" s="2" t="s">
-        <v>471</v>
+        <v>470</v>
       </c>
     </row>
     <row r="225" spans="1:2" ht="180" x14ac:dyDescent="0.25">
       <c r="A225" s="5" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="B225" s="2" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
     </row>
     <row r="226" spans="1:2" ht="60" x14ac:dyDescent="0.25">
       <c r="A226" s="5" t="s">
-        <v>470</v>
+        <v>469</v>
       </c>
       <c r="B226" s="2" t="s">
-        <v>472</v>
+        <v>471</v>
       </c>
     </row>
     <row r="227" spans="1:2" ht="117.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -6242,7 +6242,7 @@
         <v>31</v>
       </c>
       <c r="B228" s="2" t="s">
-        <v>455</v>
+        <v>454</v>
       </c>
     </row>
     <row r="229" spans="1:2" ht="45" x14ac:dyDescent="0.25">
@@ -6338,7 +6338,7 @@
         <v>67</v>
       </c>
       <c r="B240" s="2" t="s">
-        <v>498</v>
+        <v>497</v>
       </c>
     </row>
     <row r="241" spans="1:2" ht="165" x14ac:dyDescent="0.25">
@@ -6362,7 +6362,7 @@
         <v>11</v>
       </c>
       <c r="B243" s="2" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
     </row>
     <row r="244" spans="1:2" ht="180" x14ac:dyDescent="0.25">
@@ -6402,7 +6402,7 @@
         <v>5</v>
       </c>
       <c r="B248" s="2" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
     </row>
     <row r="249" spans="1:2" ht="150" x14ac:dyDescent="0.25">
@@ -6410,7 +6410,7 @@
         <v>6</v>
       </c>
       <c r="B249" s="2" t="s">
-        <v>566</v>
+        <v>565</v>
       </c>
     </row>
     <row r="250" spans="1:2" ht="255" x14ac:dyDescent="0.25">
@@ -6418,7 +6418,7 @@
         <v>7</v>
       </c>
       <c r="B250" s="2" t="s">
-        <v>594</v>
+        <v>593</v>
       </c>
     </row>
     <row r="251" spans="1:2" ht="78.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -6426,7 +6426,7 @@
         <v>8</v>
       </c>
       <c r="B251" s="2" t="s">
-        <v>565</v>
+        <v>564</v>
       </c>
     </row>
     <row r="252" spans="1:2" ht="104.65" customHeight="1" x14ac:dyDescent="0.25">
@@ -6474,7 +6474,7 @@
         <v>147</v>
       </c>
       <c r="B257" s="3" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
     </row>
     <row r="258" spans="1:2" ht="180" x14ac:dyDescent="0.25">
@@ -6482,7 +6482,7 @@
         <v>148</v>
       </c>
       <c r="B258" s="3" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
     </row>
     <row r="259" spans="1:2" ht="60" x14ac:dyDescent="0.25">
@@ -6498,7 +6498,7 @@
         <v>151</v>
       </c>
       <c r="B260" s="3" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
     </row>
     <row r="261" spans="1:2" ht="180" x14ac:dyDescent="0.25">
@@ -6506,7 +6506,7 @@
         <v>152</v>
       </c>
       <c r="B261" s="3" t="s">
-        <v>154</v>
+        <v>597</v>
       </c>
     </row>
     <row r="262" spans="1:2" ht="300" x14ac:dyDescent="0.25">
@@ -6514,303 +6514,303 @@
         <v>149</v>
       </c>
       <c r="B262" s="3" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
     </row>
     <row r="263" spans="1:2" ht="60" x14ac:dyDescent="0.25">
       <c r="A263" s="1" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="B263" s="3" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
     </row>
     <row r="264" spans="1:2" ht="240" x14ac:dyDescent="0.25">
       <c r="A264" s="1" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="B264" s="3" t="s">
-        <v>509</v>
+        <v>508</v>
       </c>
     </row>
     <row r="265" spans="1:2" ht="165" x14ac:dyDescent="0.25">
       <c r="A265" s="1" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="B265" s="3" t="s">
-        <v>508</v>
+        <v>507</v>
       </c>
     </row>
     <row r="266" spans="1:2" ht="165" x14ac:dyDescent="0.25">
       <c r="A266" s="1" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="B266" s="3" t="s">
-        <v>489</v>
+        <v>488</v>
       </c>
     </row>
     <row r="267" spans="1:2" ht="195" x14ac:dyDescent="0.25">
       <c r="A267" s="1" t="s">
-        <v>486</v>
+        <v>485</v>
       </c>
       <c r="B267" s="3" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
     </row>
     <row r="268" spans="1:2" ht="135" x14ac:dyDescent="0.25">
       <c r="A268" s="1" t="s">
-        <v>487</v>
+        <v>486</v>
       </c>
       <c r="B268" s="3" t="s">
-        <v>592</v>
+        <v>591</v>
       </c>
     </row>
     <row r="269" spans="1:2" ht="150" x14ac:dyDescent="0.25">
       <c r="A269" s="1" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="B269" s="3" t="s">
-        <v>490</v>
+        <v>489</v>
       </c>
     </row>
     <row r="270" spans="1:2" ht="75" x14ac:dyDescent="0.25">
       <c r="A270" s="1" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="B270" s="3" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="271" spans="1:2" ht="120" x14ac:dyDescent="0.25">
       <c r="A271" s="1" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="B271" s="3" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
     </row>
     <row r="272" spans="1:2" ht="195" x14ac:dyDescent="0.25">
       <c r="A272" s="1" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B272" s="3" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
     </row>
     <row r="273" spans="1:2" ht="105" x14ac:dyDescent="0.25">
       <c r="A273" s="1" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="B273" s="3" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="274" spans="1:2" ht="180" x14ac:dyDescent="0.25">
       <c r="A274" s="1" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="B274" s="3" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
     </row>
     <row r="275" spans="1:2" ht="120" x14ac:dyDescent="0.25">
       <c r="A275" s="1" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="B275" s="3" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
     </row>
     <row r="276" spans="1:2" ht="135" x14ac:dyDescent="0.25">
       <c r="A276" s="1" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="B276" s="3" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="277" spans="1:2" ht="165" x14ac:dyDescent="0.25">
       <c r="A277" s="1" t="s">
-        <v>480</v>
+        <v>479</v>
       </c>
       <c r="B277" s="3" t="s">
-        <v>589</v>
+        <v>588</v>
       </c>
     </row>
     <row r="278" spans="1:2" ht="105" x14ac:dyDescent="0.25">
       <c r="A278" s="1" t="s">
-        <v>481</v>
+        <v>480</v>
       </c>
       <c r="B278" s="3" t="s">
-        <v>483</v>
+        <v>482</v>
       </c>
     </row>
     <row r="279" spans="1:2" ht="210" x14ac:dyDescent="0.25">
       <c r="A279" s="1" t="s">
-        <v>482</v>
+        <v>481</v>
       </c>
       <c r="B279" s="3" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
     </row>
     <row r="280" spans="1:2" ht="120" x14ac:dyDescent="0.25">
       <c r="A280" s="1" t="s">
-        <v>484</v>
+        <v>483</v>
       </c>
       <c r="B280" s="3" t="s">
-        <v>563</v>
+        <v>562</v>
       </c>
     </row>
     <row r="281" spans="1:2" ht="105" x14ac:dyDescent="0.25">
       <c r="A281" s="1" t="s">
-        <v>485</v>
+        <v>484</v>
       </c>
       <c r="B281" s="3" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
     </row>
     <row r="282" spans="1:2" ht="270" x14ac:dyDescent="0.25">
       <c r="A282" s="1" t="s">
-        <v>539</v>
+        <v>538</v>
       </c>
       <c r="B282" s="3" t="s">
-        <v>554</v>
+        <v>553</v>
       </c>
     </row>
     <row r="283" spans="1:2" ht="150" x14ac:dyDescent="0.25">
       <c r="A283" s="1" t="s">
-        <v>540</v>
+        <v>539</v>
       </c>
       <c r="B283" s="3" t="s">
-        <v>549</v>
+        <v>548</v>
       </c>
     </row>
     <row r="284" spans="1:2" ht="60" x14ac:dyDescent="0.25">
       <c r="A284" s="1" t="s">
-        <v>541</v>
+        <v>540</v>
       </c>
       <c r="B284" s="3" t="s">
-        <v>555</v>
+        <v>554</v>
       </c>
     </row>
     <row r="285" spans="1:2" ht="60" x14ac:dyDescent="0.25">
       <c r="A285" s="1" t="s">
-        <v>542</v>
+        <v>541</v>
       </c>
       <c r="B285" s="3" t="s">
-        <v>550</v>
+        <v>549</v>
       </c>
     </row>
     <row r="286" spans="1:2" ht="60" x14ac:dyDescent="0.25">
       <c r="A286" s="1" t="s">
-        <v>543</v>
+        <v>542</v>
       </c>
       <c r="B286" s="3" t="s">
-        <v>552</v>
+        <v>551</v>
       </c>
     </row>
     <row r="287" spans="1:2" ht="60" x14ac:dyDescent="0.25">
       <c r="A287" s="1" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
       <c r="B287" s="3" t="s">
-        <v>551</v>
+        <v>550</v>
       </c>
     </row>
     <row r="288" spans="1:2" ht="60" x14ac:dyDescent="0.25">
       <c r="A288" s="1" t="s">
-        <v>545</v>
+        <v>544</v>
       </c>
       <c r="B288" s="3" t="s">
-        <v>553</v>
+        <v>552</v>
       </c>
     </row>
     <row r="289" spans="1:2" ht="60" x14ac:dyDescent="0.25">
       <c r="A289" s="1" t="s">
-        <v>546</v>
+        <v>545</v>
       </c>
       <c r="B289" s="3" t="s">
-        <v>556</v>
+        <v>555</v>
       </c>
     </row>
     <row r="290" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A290" s="1" t="s">
-        <v>547</v>
+        <v>546</v>
       </c>
       <c r="B290" s="3" t="s">
-        <v>557</v>
+        <v>556</v>
       </c>
     </row>
     <row r="291" spans="1:2" ht="195" x14ac:dyDescent="0.25">
       <c r="A291" s="1" t="s">
-        <v>548</v>
+        <v>547</v>
       </c>
       <c r="B291" s="3" t="s">
-        <v>558</v>
+        <v>557</v>
       </c>
     </row>
     <row r="292" spans="1:2" ht="210" x14ac:dyDescent="0.25">
       <c r="A292" s="1" t="s">
-        <v>492</v>
+        <v>491</v>
       </c>
       <c r="B292" s="3" t="s">
-        <v>595</v>
+        <v>594</v>
       </c>
     </row>
     <row r="293" spans="1:2" ht="120" x14ac:dyDescent="0.25">
       <c r="A293" s="1" t="s">
-        <v>493</v>
+        <v>492</v>
       </c>
       <c r="B293" s="3" t="s">
-        <v>576</v>
+        <v>575</v>
       </c>
     </row>
     <row r="294" spans="1:2" ht="135" x14ac:dyDescent="0.25">
       <c r="A294" s="1" t="s">
-        <v>494</v>
+        <v>493</v>
       </c>
       <c r="B294" s="3" t="s">
-        <v>577</v>
+        <v>576</v>
       </c>
     </row>
     <row r="295" spans="1:2" ht="210" x14ac:dyDescent="0.25">
       <c r="A295" s="1" t="s">
+        <v>529</v>
+      </c>
+      <c r="B295" s="3" t="s">
         <v>530</v>
-      </c>
-      <c r="B295" s="3" t="s">
-        <v>531</v>
       </c>
     </row>
     <row r="296" spans="1:2" ht="45" x14ac:dyDescent="0.25">
       <c r="A296" s="1" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="B296" s="3" t="s">
-        <v>536</v>
+        <v>535</v>
       </c>
     </row>
     <row r="297" spans="1:2" ht="45" x14ac:dyDescent="0.25">
       <c r="A297" s="1" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="B297" s="3" t="s">
-        <v>537</v>
+        <v>536</v>
       </c>
     </row>
     <row r="298" spans="1:2" ht="135" x14ac:dyDescent="0.25">
       <c r="A298" s="1" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="B298" s="3" t="s">
-        <v>538</v>
+        <v>537</v>
       </c>
     </row>
     <row r="299" spans="1:2" ht="75" x14ac:dyDescent="0.25">
       <c r="A299" s="1" t="s">
-        <v>535</v>
+        <v>534</v>
       </c>
       <c r="B299" s="3" t="s">
-        <v>559</v>
+        <v>558</v>
       </c>
     </row>
     <row r="303" spans="1:2" x14ac:dyDescent="0.25">

</xml_diff>